<commit_message>
Integrate pixelprompt as a Pipeline Summary Assistant
</commit_message>
<xml_diff>
--- a/IOS_Master_Tracker_Filled_10 (1).xlsx
+++ b/IOS_Master_Tracker_Filled_10 (1).xlsx
@@ -763,7 +763,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:AY37"/>
+  <dimension ref="A1:BJ37"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.71484375" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="15" customWidth="1" style="23" min="1" max="1"/>
@@ -1064,6 +1064,61 @@
           <t>Justified P/E</t>
         </is>
       </c>
+      <c r="AZ1" t="inlineStr">
+        <is>
+          <t>Previous Close</t>
+        </is>
+      </c>
+      <c r="BA1" t="inlineStr">
+        <is>
+          <t>Dividend Yield</t>
+        </is>
+      </c>
+      <c r="BB1" t="inlineStr">
+        <is>
+          <t>Beta</t>
+        </is>
+      </c>
+      <c r="BC1" t="inlineStr">
+        <is>
+          <t>P/E</t>
+        </is>
+      </c>
+      <c r="BD1" t="inlineStr">
+        <is>
+          <t>P/B</t>
+        </is>
+      </c>
+      <c r="BE1" t="inlineStr">
+        <is>
+          <t>Investment Confidence (%)</t>
+        </is>
+      </c>
+      <c r="BF1" t="inlineStr">
+        <is>
+          <t>Risk Score (Engine)</t>
+        </is>
+      </c>
+      <c r="BG1" t="inlineStr">
+        <is>
+          <t>Risk Confidence (%)</t>
+        </is>
+      </c>
+      <c r="BH1" t="inlineStr">
+        <is>
+          <t>Portfolio Weight</t>
+        </is>
+      </c>
+      <c r="BI1" t="inlineStr">
+        <is>
+          <t>Valuation Status</t>
+        </is>
+      </c>
+      <c r="BJ1" t="inlineStr">
+        <is>
+          <t>Overall Recommendation</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="15" customHeight="1" s="24">
       <c r="A2" s="32" t="n">
@@ -1090,7 +1145,7 @@
         </is>
       </c>
       <c r="F2" s="32" t="n">
-        <v>192259375104</v>
+        <v>192755793920</v>
       </c>
       <c r="G2" s="32" t="inlineStr">
         <is>
@@ -1103,16 +1158,16 @@
         </is>
       </c>
       <c r="I2" s="32" t="n">
-        <v>35</v>
+        <v>97</v>
       </c>
       <c r="J2" s="32" t="n">
-        <v>21.45869862932818</v>
+        <v>27.68506232955167</v>
       </c>
       <c r="K2" s="32" t="n">
         <v>97</v>
       </c>
       <c r="L2" s="32" t="n">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="M2" s="32" t="inlineStr">
         <is>
@@ -1139,7 +1194,7 @@
         <v>1.85</v>
       </c>
       <c r="S2" s="32" t="n">
-        <v>32.542988619078</v>
+        <v>32.62678849486846</v>
       </c>
       <c r="T2" s="32" t="n">
         <v>0.3603169934056724</v>
@@ -1153,7 +1208,7 @@
         </is>
       </c>
       <c r="W2" s="32" t="n">
-        <v>0.02301653570014912</v>
+        <v>2.29574191605883</v>
       </c>
       <c r="X2" s="32" t="n">
         <v>16</v>
@@ -1192,22 +1247,22 @@
         </is>
       </c>
       <c r="AH2" s="33" t="n">
-        <v>188.055041657046</v>
+        <v>229.4640886763601</v>
       </c>
       <c r="AI2" s="34" t="n">
         <v>752</v>
       </c>
       <c r="AJ2" s="33" t="n">
-        <v>235.0688020713075</v>
+        <v>286.8301108454501</v>
       </c>
       <c r="AK2" s="35" t="n">
-        <v>-2.295205459740367</v>
+        <v>-170.7526060325124</v>
       </c>
       <c r="AL2" s="32" t="n">
-        <v>0.05932203389830508</v>
+        <v>3.875698832038486</v>
       </c>
       <c r="AM2" s="36" t="n">
-        <v>59322.03389830508</v>
+        <v>38756.98832038486</v>
       </c>
       <c r="AN2" s="32" t="inlineStr">
         <is>
@@ -1255,13 +1310,38 @@
         </is>
       </c>
       <c r="AW2" s="37" t="n">
-        <v>18.93000088418207</v>
+        <v>19.17000020858422</v>
       </c>
       <c r="AX2" s="38" t="n">
-        <v>0.1</v>
+        <v>13.813758</v>
       </c>
       <c r="AY2" s="38" t="n">
-        <v>12.2240666703748</v>
+        <v>14.96244709678926</v>
+      </c>
+      <c r="BA2" t="n">
+        <v>1.58</v>
+      </c>
+      <c r="BC2" t="n">
+        <v>40.511215</v>
+      </c>
+      <c r="BE2" t="n">
+        <v>100</v>
+      </c>
+      <c r="BF2" t="n">
+        <v>42.91739725865636</v>
+      </c>
+      <c r="BG2" t="n">
+        <v>100</v>
+      </c>
+      <c r="BI2" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="BJ2" t="inlineStr">
+        <is>
+          <t>Avoid</t>
+        </is>
       </c>
     </row>
     <row r="3" ht="15" customHeight="1" s="24">
@@ -1289,7 +1369,7 @@
         </is>
       </c>
       <c r="F3" s="32" t="n">
-        <v>7671792009216</v>
+        <v>7583873630208</v>
       </c>
       <c r="G3" s="32" t="inlineStr">
         <is>
@@ -1302,16 +1382,16 @@
         </is>
       </c>
       <c r="I3" s="32" t="n">
-        <v>32</v>
+        <v>74</v>
       </c>
       <c r="J3" s="32" t="n">
-        <v>3.120356201257398</v>
+        <v>71.24414456138504</v>
       </c>
       <c r="K3" s="32" t="n">
         <v>95</v>
       </c>
       <c r="L3" s="32" t="n">
-        <v>90</v>
+        <v>100</v>
       </c>
       <c r="M3" s="32" t="inlineStr">
         <is>
@@ -1338,7 +1418,7 @@
         <v>1.66</v>
       </c>
       <c r="S3" s="32" t="n">
-        <v>11.53793084243383</v>
+        <v>11.4067524547283</v>
       </c>
       <c r="T3" s="32" t="n">
         <v>0.4536403694758384</v>
@@ -1350,7 +1430,7 @@
         <v>0.11</v>
       </c>
       <c r="W3" s="32" t="n">
-        <v>0.06200478154119719</v>
+        <v>6.271784052138364</v>
       </c>
       <c r="X3" s="32" t="n">
         <v>6</v>
@@ -1389,22 +1469,22 @@
         </is>
       </c>
       <c r="AH3" s="33" t="n">
-        <v/>
+        <v>2307.254170003561</v>
       </c>
       <c r="AI3" s="34" t="n">
         <v>1983</v>
       </c>
       <c r="AJ3" s="33" t="n">
-        <v/>
+        <v>2884.067712504452</v>
       </c>
       <c r="AK3" s="35" t="n">
-        <v/>
+        <v>27.32140126558265</v>
       </c>
       <c r="AL3" s="32" t="n">
-        <v>0.05423728813559322</v>
+        <v>9.973640101629945</v>
       </c>
       <c r="AM3" s="36" t="n">
-        <v>54237.28813559322</v>
+        <v>99736.40101629945</v>
       </c>
       <c r="AN3" s="32" t="inlineStr">
         <is>
@@ -1452,14 +1532,38 @@
         </is>
       </c>
       <c r="AW3" s="37" t="n">
-        <v>133.7589331881477</v>
+        <v>133.7399958195484</v>
       </c>
       <c r="AX3" s="38" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="AY3" s="38">
-        <f>IFERROR(IF(OR(T3="",T3=0,AW3="",T3-AX3&lt;3),"N/A",ROUND((1-(AX3/T3))*100/(Dashboard!$B$14-AX3),1)),"N/A")</f>
-        <v/>
+        <v>25</v>
+      </c>
+      <c r="AY3" s="38" t="n">
+        <v>21.56473540081091</v>
+      </c>
+      <c r="BA3" t="n">
+        <v>6.03</v>
+      </c>
+      <c r="BC3" t="n">
+        <v>15.672948</v>
+      </c>
+      <c r="BE3" t="n">
+        <v>100</v>
+      </c>
+      <c r="BF3" t="n">
+        <v>24.38359139004868</v>
+      </c>
+      <c r="BG3" t="n">
+        <v>100</v>
+      </c>
+      <c r="BI3" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="BJ3" t="inlineStr">
+        <is>
+          <t>Buy</t>
+        </is>
       </c>
     </row>
     <row r="4" ht="15" customHeight="1" s="24">
@@ -1487,7 +1591,7 @@
         </is>
       </c>
       <c r="F4" s="32" t="n">
-        <v>1142075424768</v>
+        <v>1138600443904</v>
       </c>
       <c r="G4" s="32" t="inlineStr">
         <is>
@@ -1500,16 +1604,16 @@
         </is>
       </c>
       <c r="I4" s="32" t="n">
-        <v>32</v>
+        <v>94</v>
       </c>
       <c r="J4" s="32" t="n">
-        <v>28.81633447147184</v>
+        <v>44.81831730859492</v>
       </c>
       <c r="K4" s="32" t="n">
         <v>94</v>
       </c>
       <c r="L4" s="32" t="n">
-        <v>87</v>
+        <v>100</v>
       </c>
       <c r="M4" s="32" t="inlineStr">
         <is>
@@ -1536,7 +1640,7 @@
         <v>0.5600000000000001</v>
       </c>
       <c r="S4" s="32" t="n">
-        <v>7.950194085688558</v>
+        <v>7.926525036910297</v>
       </c>
       <c r="T4" s="32" t="n">
         <v>0.2368743551054329</v>
@@ -1548,7 +1652,7 @@
         <v>0.29</v>
       </c>
       <c r="W4" s="32" t="n">
-        <v>0.04523304132926451</v>
+        <v>4.53681097301875</v>
       </c>
       <c r="X4" s="32" t="n">
         <v>23</v>
@@ -1587,22 +1691,22 @@
         </is>
       </c>
       <c r="AH4" s="33" t="n">
-        <v>1275.801572118107</v>
+        <v>2080.023350647083</v>
       </c>
       <c r="AI4" s="34" t="n">
         <v>2476</v>
       </c>
       <c r="AJ4" s="33" t="n">
-        <v>1594.751965147634</v>
+        <v>2600.029188308853</v>
       </c>
       <c r="AK4" s="35" t="n">
-        <v>-0.566262374706506</v>
+        <v>4.224152128857054</v>
       </c>
       <c r="AL4" s="32" t="n">
-        <v>0.05423728813559322</v>
+        <v>6.274224633456496</v>
       </c>
       <c r="AM4" s="36" t="n">
-        <v>54237.28813559322</v>
+        <v>62742.24633456496</v>
       </c>
       <c r="AN4" s="32" t="inlineStr">
         <is>
@@ -1650,13 +1754,38 @@
         </is>
       </c>
       <c r="AW4" s="37" t="n">
-        <v>117.1100019621481</v>
+        <v>116.3600055773553</v>
       </c>
       <c r="AX4" s="38" t="n">
-        <v>0.1</v>
+        <v>24.1328883</v>
       </c>
       <c r="AY4" s="38" t="n">
-        <v>13.65954574002256</v>
+        <v>22.34469910887636</v>
+      </c>
+      <c r="BA4" t="n">
+        <v>0.48</v>
+      </c>
+      <c r="BC4" t="n">
+        <v>21.400824</v>
+      </c>
+      <c r="BE4" t="n">
+        <v>100</v>
+      </c>
+      <c r="BF4" t="n">
+        <v>54.25334723985804</v>
+      </c>
+      <c r="BG4" t="n">
+        <v>100</v>
+      </c>
+      <c r="BI4" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="BJ4" t="inlineStr">
+        <is>
+          <t>Hold</t>
+        </is>
       </c>
     </row>
     <row r="5" ht="15" customHeight="1" s="24">
@@ -1684,7 +1813,7 @@
         </is>
       </c>
       <c r="F5" s="32" t="n">
-        <v>80317308928</v>
+        <v>80563920896</v>
       </c>
       <c r="G5" s="32" t="inlineStr">
         <is>
@@ -1697,16 +1826,16 @@
         </is>
       </c>
       <c r="I5" s="32" t="n">
-        <v>10</v>
+        <v>45</v>
       </c>
       <c r="J5" s="32" t="n">
-        <v>22.72044639936992</v>
+        <v>12.27579912028354</v>
       </c>
       <c r="K5" s="32" t="n">
         <v>92</v>
       </c>
       <c r="L5" s="32" t="n">
-        <v>90</v>
+        <v>100</v>
       </c>
       <c r="M5" s="32" t="inlineStr">
         <is>
@@ -1784,22 +1913,22 @@
         </is>
       </c>
       <c r="AH5" s="33" t="n">
-        <v>365.4915545718279</v>
+        <v>384.7243580124707</v>
       </c>
       <c r="AI5" s="34" t="n">
         <v>1149</v>
       </c>
       <c r="AJ5" s="33" t="n">
-        <v>456.8644432147848</v>
+        <v>480.9054475155883</v>
       </c>
       <c r="AK5" s="35" t="n">
-        <v>-1.495050811962841</v>
+        <v>-137.7598353079453</v>
       </c>
       <c r="AL5" s="32" t="n">
-        <v>0.01694915254237288</v>
+        <v>1.718518807957924</v>
       </c>
       <c r="AM5" s="36" t="n">
-        <v>16949.15254237288</v>
+        <v>17185.18807957924</v>
       </c>
       <c r="AN5" s="32" t="inlineStr">
         <is>
@@ -1850,10 +1979,35 @@
         <v>58.61999611942723</v>
       </c>
       <c r="AX5" s="38" t="n">
-        <v>0.1</v>
+        <v>13.044297</v>
       </c>
       <c r="AY5" s="38" t="n">
-        <v>7.798983325619407</v>
+        <v>8.203777678532726</v>
+      </c>
+      <c r="BA5" t="n">
+        <v>0.61</v>
+      </c>
+      <c r="BC5" t="n">
+        <v>19.50529</v>
+      </c>
+      <c r="BE5" t="n">
+        <v>100</v>
+      </c>
+      <c r="BF5" t="n">
+        <v>45.44089279873983</v>
+      </c>
+      <c r="BG5" t="n">
+        <v>100</v>
+      </c>
+      <c r="BI5" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="BJ5" t="inlineStr">
+        <is>
+          <t>Avoid</t>
+        </is>
       </c>
     </row>
     <row r="6" ht="15" customHeight="1" s="24">
@@ -1881,7 +2035,7 @@
         </is>
       </c>
       <c r="F6" s="32" t="n">
-        <v>750143340544</v>
+        <v>763157348352</v>
       </c>
       <c r="G6" s="32" t="inlineStr">
         <is>
@@ -1894,10 +2048,10 @@
         </is>
       </c>
       <c r="I6" s="32" t="n">
-        <v>27.5</v>
+        <v>85</v>
       </c>
       <c r="J6" s="32" t="n">
-        <v>1.827469377782569</v>
+        <v>23.94665102888482</v>
       </c>
       <c r="K6" s="32" t="inlineStr">
         <is>
@@ -1905,7 +2059,7 @@
         </is>
       </c>
       <c r="L6" s="32" t="n">
-        <v>85</v>
+        <v>100</v>
       </c>
       <c r="M6" s="32" t="inlineStr">
         <is>
@@ -1932,7 +2086,7 @@
         <v>1.04</v>
       </c>
       <c r="S6" s="32" t="n">
-        <v>31.10431965920068</v>
+        <v>31.64827142031346</v>
       </c>
       <c r="T6" s="32" t="n">
         <v>0.2379630651498401</v>
@@ -1944,7 +2098,7 @@
         <v>0.06</v>
       </c>
       <c r="W6" s="32" t="n">
-        <v>0.0209434911961649</v>
+        <v>2.058352686292514</v>
       </c>
       <c r="X6" s="32" t="n">
         <v>19.6</v>
@@ -1983,22 +2137,22 @@
         </is>
       </c>
       <c r="AH6" s="33" t="n">
-        <v/>
+        <v>1583.048870839265</v>
       </c>
       <c r="AI6" s="34" t="n">
         <v>4683</v>
       </c>
       <c r="AJ6" s="33" t="n">
-        <v/>
+        <v>1978.811088549081</v>
       </c>
       <c r="AK6" s="35" t="n">
-        <v/>
+        <v>-146.8552975201725</v>
       </c>
       <c r="AL6" s="39" t="n">
-        <v>0.04661016949152542</v>
+        <v>3.35234959268322</v>
       </c>
       <c r="AM6" s="36" t="n">
-        <v>46610.16949152543</v>
+        <v>33523.4959268322</v>
       </c>
       <c r="AN6" s="32" t="inlineStr">
         <is>
@@ -2049,11 +2203,35 @@
         <v>119.7800029386826</v>
       </c>
       <c r="AX6" s="38" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="AY6" s="38">
-        <f>IFERROR(IF(OR(T6="",T6=0,AW6="",T6-AX6&lt;3),"N/A",ROUND((1-(AX6/T6))*100/(Dashboard!$B$14-AX6),1)),"N/A")</f>
-        <v/>
+        <v>18.14655820438004</v>
+      </c>
+      <c r="AY6" s="38" t="n">
+        <v>16.52037976748273</v>
+      </c>
+      <c r="BA6" t="n">
+        <v>0.93</v>
+      </c>
+      <c r="BC6" t="n">
+        <v>40.781433</v>
+      </c>
+      <c r="BE6" t="n">
+        <v>100</v>
+      </c>
+      <c r="BF6" t="n">
+        <v>43.65493875556514</v>
+      </c>
+      <c r="BG6" t="n">
+        <v>100</v>
+      </c>
+      <c r="BI6" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="BJ6" t="inlineStr">
+        <is>
+          <t>Avoid</t>
+        </is>
       </c>
     </row>
     <row r="7" ht="15" customHeight="1" s="24">
@@ -2081,7 +2259,7 @@
         </is>
       </c>
       <c r="F7" s="32" t="n">
-        <v>253774807040</v>
+        <v>247757602816</v>
       </c>
       <c r="G7" s="32" t="inlineStr">
         <is>
@@ -2094,16 +2272,16 @@
         </is>
       </c>
       <c r="I7" s="39" t="n">
-        <v>24.5</v>
+        <v>58.5</v>
       </c>
       <c r="J7" s="39" t="n">
-        <v>3.927452762874952</v>
+        <v>15.25244013371815</v>
       </c>
       <c r="K7" s="32" t="n">
         <v>70</v>
       </c>
       <c r="L7" s="32" t="n">
-        <v>65</v>
+        <v>100</v>
       </c>
       <c r="M7" s="32" t="inlineStr">
         <is>
@@ -2181,22 +2359,22 @@
         </is>
       </c>
       <c r="AH7" s="33" t="n">
-        <v/>
+        <v>193.1058491092882</v>
       </c>
       <c r="AI7" s="34" t="n">
         <v>2450</v>
       </c>
       <c r="AJ7" s="33" t="n">
-        <v/>
+        <v>241.3823113866103</v>
       </c>
       <c r="AK7" s="35" t="n">
-        <v/>
+        <v>-807.4815745266367</v>
       </c>
       <c r="AL7" s="39" t="n">
-        <v>0.04152542372881356</v>
+        <v>2.13522598245657</v>
       </c>
       <c r="AM7" s="36" t="n">
-        <v>41525.42372881356</v>
+        <v>21352.25982456571</v>
       </c>
       <c r="AN7" s="32" t="inlineStr">
         <is>
@@ -2244,14 +2422,38 @@
         </is>
       </c>
       <c r="AW7" s="37" t="n">
-        <v>43.59000158005741</v>
+        <v>43.61000017818284</v>
       </c>
       <c r="AX7" s="38" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="AY7" s="38">
-        <f>IFERROR(IF(OR(T7="",T7=0,AW7="",T7-AX7&lt;3),"N/A",ROUND((1-(AX7/T7))*100/(Dashboard!$B$14-AX7),1)),"N/A")</f>
-        <v/>
+        <v>17.2376802</v>
+      </c>
+      <c r="AY7" s="38" t="n">
+        <v>5.535022045095397</v>
+      </c>
+      <c r="BA7" t="n">
+        <v>0.48</v>
+      </c>
+      <c r="BC7" t="n">
+        <v>50.229305</v>
+      </c>
+      <c r="BE7" t="n">
+        <v>100</v>
+      </c>
+      <c r="BF7" t="n">
+        <v>47.85490552574991</v>
+      </c>
+      <c r="BG7" t="n">
+        <v>100</v>
+      </c>
+      <c r="BI7" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="BJ7" t="inlineStr">
+        <is>
+          <t>Avoid</t>
+        </is>
       </c>
     </row>
     <row r="8" ht="15" customHeight="1" s="24">
@@ -2279,7 +2481,7 @@
         </is>
       </c>
       <c r="F8" s="32" t="n">
-        <v>1513511976960</v>
+        <v>1516699779072</v>
       </c>
       <c r="G8" s="32" t="inlineStr">
         <is>
@@ -2292,16 +2494,16 @@
         </is>
       </c>
       <c r="I8" s="39" t="n">
-        <v>27.5</v>
+        <v>89.5</v>
       </c>
       <c r="J8" s="39" t="n">
-        <v>20.12923649819</v>
+        <v>26.73433333411995</v>
       </c>
       <c r="K8" s="32" t="n">
         <v>80</v>
       </c>
       <c r="L8" s="32" t="n">
-        <v>70</v>
+        <v>100</v>
       </c>
       <c r="M8" s="32" t="inlineStr">
         <is>
@@ -2328,7 +2530,7 @@
         <v>2.05</v>
       </c>
       <c r="S8" s="32" t="n">
-        <v>62.96563427546059</v>
+        <v>63.09866167596553</v>
       </c>
       <c r="T8" s="32" t="n">
         <v>0.2786673053960043</v>
@@ -2340,7 +2542,7 @@
         <v>0.003</v>
       </c>
       <c r="W8" s="32" t="n">
-        <v>0.009825519393814054</v>
+        <v>0.9804804797515924</v>
       </c>
       <c r="X8" s="32" t="n">
         <v>13</v>
@@ -2379,22 +2581,22 @@
         </is>
       </c>
       <c r="AH8" s="33" t="n">
-        <v>685.9587250582365</v>
+        <v>756.8694949111471</v>
       </c>
       <c r="AI8" s="34" t="n">
         <v>5478</v>
       </c>
       <c r="AJ8" s="33" t="n">
-        <v>857.4484063227956</v>
+        <v>946.0868686389338</v>
       </c>
       <c r="AK8" s="35" t="n">
-        <v>-5.367730069515722</v>
+        <v>-478.3295573979848</v>
       </c>
       <c r="AL8" s="39" t="n">
-        <v>0.04661016949152542</v>
+        <v>3.74260398062301</v>
       </c>
       <c r="AM8" s="36" t="n">
-        <v>46610.16949152543</v>
+        <v>37426.0398062301</v>
       </c>
       <c r="AN8" s="32" t="inlineStr">
         <is>
@@ -2445,10 +2647,35 @@
         <v>85.46000129160427</v>
       </c>
       <c r="AX8" s="38" t="n">
-        <v>0.1</v>
+        <v>10.9602055</v>
       </c>
       <c r="AY8" s="38" t="n">
-        <v>10.06394843101873</v>
+        <v>11.07052268475233</v>
+      </c>
+      <c r="BA8" t="n">
+        <v>1.18</v>
+      </c>
+      <c r="BC8" t="n">
+        <v>64.02410999999999</v>
+      </c>
+      <c r="BE8" t="n">
+        <v>100</v>
+      </c>
+      <c r="BF8" t="n">
+        <v>40.25847299638001</v>
+      </c>
+      <c r="BG8" t="n">
+        <v>100</v>
+      </c>
+      <c r="BI8" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="BJ8" t="inlineStr">
+        <is>
+          <t>Avoid</t>
+        </is>
       </c>
     </row>
     <row r="9" ht="15" customHeight="1" s="24">
@@ -2476,7 +2703,7 @@
         </is>
       </c>
       <c r="F9" s="32" t="n">
-        <v>212548780032</v>
+        <v>215517085696</v>
       </c>
       <c r="G9" s="32" t="inlineStr">
         <is>
@@ -2489,16 +2716,16 @@
         </is>
       </c>
       <c r="I9" s="32" t="n">
-        <v>7</v>
+        <v>44.5</v>
       </c>
       <c r="J9" s="32" t="n">
-        <v>13.73344096126002</v>
+        <v>7.238618772239289</v>
       </c>
       <c r="K9" s="32" t="n">
         <v>55</v>
       </c>
       <c r="L9" s="32" t="n">
-        <v>45</v>
+        <v>100</v>
       </c>
       <c r="M9" s="32" t="inlineStr">
         <is>
@@ -2525,7 +2752,7 @@
         <v>2.49</v>
       </c>
       <c r="S9" s="32" t="n">
-        <v>158.8360123893935</v>
+        <v>161.015689190122</v>
       </c>
       <c r="T9" s="32" t="n">
         <v>0.1143100972906209</v>
@@ -2537,7 +2764,7 @@
         <v>0.3</v>
       </c>
       <c r="W9" s="32" t="n">
-        <v>0.002926430507452547</v>
+        <v>0.2886815282885787</v>
       </c>
       <c r="X9" s="32" t="n">
         <v>29.6</v>
@@ -2576,22 +2803,22 @@
         </is>
       </c>
       <c r="AH9" s="33" t="n">
-        <v/>
+        <v>352.3733223219795</v>
       </c>
       <c r="AI9" s="34" t="n">
         <v>7034</v>
       </c>
       <c r="AJ9" s="33" t="n">
-        <v/>
+        <v>440.4666529024743</v>
       </c>
       <c r="AK9" s="35" t="n">
-        <v/>
+        <v>-1490.699308070285</v>
       </c>
       <c r="AL9" s="39" t="n">
-        <v>0.01186440677966102</v>
+        <v>1.013351748577912</v>
       </c>
       <c r="AM9" s="36" t="n">
-        <v>11864.40677966102</v>
+        <v>10133.51748577912</v>
       </c>
       <c r="AN9" s="32" t="inlineStr">
         <is>
@@ -2639,14 +2866,35 @@
         </is>
       </c>
       <c r="AW9" s="37" t="n">
-        <v>30.23999880965562</v>
+        <v>30.29999918265898</v>
       </c>
       <c r="AX9" s="38" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="AY9" s="38">
-        <f>IFERROR(IF(OR(T9="",T9=0,AW9="",T9-AX9&lt;3),"N/A",ROUND((1-(AX9/T9))*100/(Dashboard!$B$14-AX9),1)),"N/A")</f>
-        <v/>
+        <v>12.121</v>
+      </c>
+      <c r="AY9" s="38" t="n">
+        <v>14.53685323110476</v>
+      </c>
+      <c r="BC9" t="n">
+        <v>231.23763</v>
+      </c>
+      <c r="BE9" t="n">
+        <v>100</v>
+      </c>
+      <c r="BF9" t="n">
+        <v>67.46688192252005</v>
+      </c>
+      <c r="BG9" t="n">
+        <v>100</v>
+      </c>
+      <c r="BI9" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="BJ9" t="inlineStr">
+        <is>
+          <t>Avoid</t>
+        </is>
       </c>
     </row>
     <row r="10" ht="15" customHeight="1" s="24">
@@ -2674,7 +2922,7 @@
         </is>
       </c>
       <c r="F10" s="32" t="n">
-        <v>492909330432</v>
+        <v>485678678016</v>
       </c>
       <c r="G10" s="32" t="inlineStr">
         <is>
@@ -2687,16 +2935,16 @@
         </is>
       </c>
       <c r="I10" s="39" t="n">
-        <v>7</v>
+        <v>27.5</v>
       </c>
       <c r="J10" s="39" t="n">
-        <v>14.17277603730283</v>
+        <v>4.352486589741723</v>
       </c>
       <c r="K10" s="32" t="n">
         <v>55</v>
       </c>
       <c r="L10" s="32" t="n">
-        <v>60</v>
+        <v>100</v>
       </c>
       <c r="M10" s="32" t="inlineStr">
         <is>
@@ -2723,7 +2971,7 @@
         <v>1.13</v>
       </c>
       <c r="S10" s="32" t="n">
-        <v>42.84014997101866</v>
+        <v>42.26286620009102</v>
       </c>
       <c r="T10" s="32" t="n">
         <v>0.1022446814323704</v>
@@ -2735,7 +2983,7 @@
         <v>0.1</v>
       </c>
       <c r="W10" s="32" t="n">
-        <v>0.02249053471899838</v>
+        <v>2.279774106490244</v>
       </c>
       <c r="X10" s="32" t="n">
         <v>-0.1</v>
@@ -2774,22 +3022,22 @@
         </is>
       </c>
       <c r="AH10" s="33" t="n">
-        <v/>
+        <v>435.8911504473959</v>
       </c>
       <c r="AI10" s="34" t="n">
         <v>1325</v>
       </c>
       <c r="AJ10" s="33" t="n">
-        <v/>
+        <v>544.8639380592449</v>
       </c>
       <c r="AK10" s="35" t="n">
-        <v/>
+        <v>-153.9533089542707</v>
       </c>
       <c r="AL10" s="39" t="n">
-        <v>0.01186440677966102</v>
+        <v>0.6093151242184088</v>
       </c>
       <c r="AM10" s="36" t="n">
-        <v>11864.40677966102</v>
+        <v>6093.151242184089</v>
       </c>
       <c r="AN10" s="32" t="inlineStr">
         <is>
@@ -2837,14 +3085,38 @@
         </is>
       </c>
       <c r="AW10" s="37" t="n">
-        <v>27.19999972108524</v>
+        <v>25.64999957364314</v>
       </c>
       <c r="AX10" s="38" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="AY10" s="38">
-        <f>IFERROR(IF(OR(T10="",T10=0,AW10="",T10-AX10&lt;3),"N/A",ROUND((1-(AX10/T10))*100/(Dashboard!$B$14-AX10),1)),"N/A")</f>
-        <v/>
+        <v>10.48834958223998</v>
+      </c>
+      <c r="AY10" s="38" t="n">
+        <v>21.24225879373274</v>
+      </c>
+      <c r="BA10" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="BC10" t="n">
+        <v>53.94542</v>
+      </c>
+      <c r="BE10" t="n">
+        <v>100</v>
+      </c>
+      <c r="BF10" t="n">
+        <v>68.34555207460565</v>
+      </c>
+      <c r="BG10" t="n">
+        <v>100</v>
+      </c>
+      <c r="BI10" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="BJ10" t="inlineStr">
+        <is>
+          <t>Avoid</t>
+        </is>
       </c>
     </row>
     <row r="11" ht="15" customHeight="1" s="24">
@@ -2872,7 +3144,7 @@
         </is>
       </c>
       <c r="F11" s="32" t="n">
-        <v>244973895680</v>
+        <v>242484903936</v>
       </c>
       <c r="G11" s="32" t="inlineStr">
         <is>
@@ -2885,16 +3157,16 @@
         </is>
       </c>
       <c r="I11" s="39" t="n">
-        <v>24.5</v>
+        <v>73.5</v>
       </c>
       <c r="J11" s="39" t="n">
-        <v>24.82171067930616</v>
+        <v>18.50604265070997</v>
       </c>
       <c r="K11" s="32" t="n">
         <v>70</v>
       </c>
       <c r="L11" s="32" t="n">
-        <v>60</v>
+        <v>100</v>
       </c>
       <c r="M11" s="32" t="inlineStr">
         <is>
@@ -2921,7 +3193,7 @@
         <v>1.66</v>
       </c>
       <c r="S11" s="32" t="n">
-        <v>51.20987328027297</v>
+        <v>50.69429607652525</v>
       </c>
       <c r="T11" s="32" t="n">
         <v>0.1941870698690816</v>
@@ -2933,7 +3205,7 @@
         <v>0.4</v>
       </c>
       <c r="W11" s="32" t="n">
-        <v>-0.00204076197782774</v>
+        <v>-0.2061517179802629</v>
       </c>
       <c r="X11" s="32" t="n">
         <v>37</v>
@@ -2972,22 +3244,22 @@
         </is>
       </c>
       <c r="AH11" s="33" t="n">
-        <v>942.3665521546717</v>
+        <v>904.6808310954592</v>
       </c>
       <c r="AI11" s="34" t="n">
         <v>18944</v>
       </c>
       <c r="AJ11" s="33" t="n">
-        <v>1177.95819019334</v>
+        <v>1130.851038869324</v>
       </c>
       <c r="AK11" s="35" t="n">
-        <v>-15.20940383025486</v>
+        <v>-1571.307656833129</v>
       </c>
       <c r="AL11" s="39" t="n">
-        <v>0.04152542372881356</v>
+        <v>2.5907056676716</v>
       </c>
       <c r="AM11" s="36" t="n">
-        <v>41525.42372881356</v>
+        <v>25907.056676716</v>
       </c>
       <c r="AN11" s="32" t="inlineStr">
         <is>
@@ -3035,13 +3307,38 @@
         </is>
       </c>
       <c r="AW11" s="37" t="n">
-        <v>284.1600181348084</v>
+        <v>284.3399972197867</v>
       </c>
       <c r="AX11" s="38" t="n">
         <v>0.1</v>
       </c>
       <c r="AY11" s="38" t="n">
-        <v>4.151979804001761</v>
+        <v>3.977108528062615</v>
+      </c>
+      <c r="BA11" t="n">
+        <v>0.18</v>
+      </c>
+      <c r="BC11" t="n">
+        <v>66.46972</v>
+      </c>
+      <c r="BE11" t="n">
+        <v>100</v>
+      </c>
+      <c r="BF11" t="n">
+        <v>49.64342135861233</v>
+      </c>
+      <c r="BG11" t="n">
+        <v>100</v>
+      </c>
+      <c r="BI11" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="BJ11" t="inlineStr">
+        <is>
+          <t>Avoid</t>
+        </is>
       </c>
     </row>
     <row r="12" ht="15" customHeight="1" s="24">
@@ -3069,7 +3366,7 @@
         </is>
       </c>
       <c r="F12" s="32" t="n">
-        <v>116990902272</v>
+        <v>114275663872</v>
       </c>
       <c r="G12" s="32" t="inlineStr">
         <is>
@@ -3082,16 +3379,16 @@
         </is>
       </c>
       <c r="I12" s="39" t="n">
-        <v>7</v>
+        <v>44.5</v>
       </c>
       <c r="J12" s="39" t="n">
-        <v>23.54731268133384</v>
+        <v>11.77144585680644</v>
       </c>
       <c r="K12" s="32" t="n">
         <v>70</v>
       </c>
       <c r="L12" s="32" t="n">
-        <v>60</v>
+        <v>100</v>
       </c>
       <c r="M12" s="32" t="inlineStr">
         <is>
@@ -3118,7 +3415,7 @@
         <v>1.85</v>
       </c>
       <c r="S12" s="32" t="n">
-        <v>27.50078110585549</v>
+        <v>26.86810911107487</v>
       </c>
       <c r="T12" s="32" t="n">
         <v>0.1479510631746486</v>
@@ -3130,7 +3427,7 @@
         <v>0.12</v>
       </c>
       <c r="W12" s="32" t="n">
-        <v>0.01649649068308329</v>
+        <v>1.688493884756704</v>
       </c>
       <c r="X12" s="32" t="n">
         <v>17.5</v>
@@ -3169,22 +3466,22 @@
         </is>
       </c>
       <c r="AH12" s="33" t="n">
-        <v>136.5881214204845</v>
+        <v>156.7548939495195</v>
       </c>
       <c r="AI12" s="34" t="n">
         <v>529</v>
       </c>
       <c r="AJ12" s="33" t="n">
-        <v>170.7351517756056</v>
+        <v>195.9436174368994</v>
       </c>
       <c r="AK12" s="35" t="n">
-        <v>-2.053559823961745</v>
+        <v>-159.8961919053047</v>
       </c>
       <c r="AL12" s="39" t="n">
-        <v>0.01186440677966102</v>
+        <v>1.647913174821731</v>
       </c>
       <c r="AM12" s="36" t="n">
-        <v>11864.40677966102</v>
+        <v>16479.13174821731</v>
       </c>
       <c r="AN12" s="32" t="inlineStr">
         <is>
@@ -3232,13 +3529,38 @@
         </is>
       </c>
       <c r="AW12" s="37" t="n">
-        <v>15.34999972029347</v>
+        <v>15.19000028187629</v>
       </c>
       <c r="AX12" s="38" t="n">
-        <v>0.1</v>
+        <v>13.76500855851</v>
       </c>
       <c r="AY12" s="38" t="n">
-        <v>11.2325757747109</v>
+        <v>12.89951398531266</v>
+      </c>
+      <c r="BA12" t="n">
+        <v>0.38</v>
+      </c>
+      <c r="BC12" t="n">
+        <v>33.525345</v>
+      </c>
+      <c r="BE12" t="n">
+        <v>100</v>
+      </c>
+      <c r="BF12" t="n">
+        <v>47.09462536266767</v>
+      </c>
+      <c r="BG12" t="n">
+        <v>100</v>
+      </c>
+      <c r="BI12" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="BJ12" t="inlineStr">
+        <is>
+          <t>Avoid</t>
+        </is>
       </c>
     </row>
     <row r="13" ht="15" customHeight="1" s="24">
@@ -3266,7 +3588,7 @@
         </is>
       </c>
       <c r="F13" s="32" t="n">
-        <v>9625688604672</v>
+        <v>9582303772672</v>
       </c>
       <c r="G13" s="32" t="inlineStr">
         <is>
@@ -3279,16 +3601,16 @@
         </is>
       </c>
       <c r="I13" s="39" t="n">
+        <v>23.33333333333334</v>
+      </c>
+      <c r="J13" s="39" t="n">
         <v>0</v>
-      </c>
-      <c r="J13" s="39" t="n">
-        <v>50</v>
       </c>
       <c r="K13" s="32" t="n">
         <v>75</v>
       </c>
       <c r="L13" s="32" t="n">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="M13" s="32" t="inlineStr">
         <is>
@@ -3325,7 +3647,7 @@
         <v>1.33</v>
       </c>
       <c r="W13" s="32" t="n">
-        <v>0.02856015562939206</v>
+        <v>2.867966802884247</v>
       </c>
       <c r="X13" s="32" t="n">
         <v>5.2</v>
@@ -3364,16 +3686,16 @@
         </is>
       </c>
       <c r="AH13" s="33" t="n">
-        <v>700.9779087864911</v>
+        <v>759.0485579804152</v>
       </c>
       <c r="AI13" s="34" t="n">
         <v>1040</v>
       </c>
       <c r="AJ13" s="33" t="n">
-        <v>876.2223859831138</v>
+        <v>948.810697475519</v>
       </c>
       <c r="AK13" s="35" t="n">
-        <v>-0.1901088315952891</v>
+        <v>-9.410655124573442</v>
       </c>
       <c r="AL13" s="39">
         <f>IF(H13="Fail","Not Eligible (Failed Gate)",IF(J13="","Pending Score",IF(J13&gt;=90,"10%",IF(J13&gt;=80,"7.5%",IF(J13&gt;=70,"5%","Watchlist only")))))</f>
@@ -3429,13 +3751,38 @@
         </is>
       </c>
       <c r="AW13" s="37" t="n">
-        <v>91.20999132507966</v>
+        <v>91.01000680492893</v>
       </c>
       <c r="AX13" s="38" t="n">
-        <v>0.1</v>
+        <v>12.7778112</v>
       </c>
       <c r="AY13" s="38" t="n">
-        <v>9.611917353917439</v>
+        <v>10.42534553868277</v>
+      </c>
+      <c r="BA13" t="n">
+        <v>1.67</v>
+      </c>
+      <c r="BC13" t="n">
+        <v>11.406438</v>
+      </c>
+      <c r="BE13" t="n">
+        <v>60</v>
+      </c>
+      <c r="BF13" t="n">
+        <v>100</v>
+      </c>
+      <c r="BG13" t="n">
+        <v>100</v>
+      </c>
+      <c r="BI13" t="inlineStr">
+        <is>
+          <t>Missing EV/EBIT (EBIT &lt;= 0)</t>
+        </is>
+      </c>
+      <c r="BJ13" t="inlineStr">
+        <is>
+          <t>Avoid</t>
+        </is>
       </c>
     </row>
     <row r="14" ht="15" customHeight="1" s="24">
@@ -3463,7 +3810,7 @@
         </is>
       </c>
       <c r="F14" s="32" t="n">
-        <v>4090609270784</v>
+        <v>4084133789696</v>
       </c>
       <c r="G14" s="32" t="inlineStr">
         <is>
@@ -3476,16 +3823,16 @@
         </is>
       </c>
       <c r="I14" s="39" t="n">
-        <v>25</v>
+        <v>72</v>
       </c>
       <c r="J14" s="39" t="n">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="K14" s="32" t="n">
         <v>50</v>
       </c>
       <c r="L14" s="32" t="n">
-        <v>55</v>
+        <v>100</v>
       </c>
       <c r="M14" s="32" t="inlineStr">
         <is>
@@ -3563,16 +3910,16 @@
         </is>
       </c>
       <c r="AH14" s="33" t="n">
-        <v>566.1438216608158</v>
+        <v>959.1145637321993</v>
       </c>
       <c r="AI14" s="34" t="n">
         <v>3550</v>
       </c>
       <c r="AJ14" s="33" t="n">
-        <v>707.6797770760197</v>
+        <v>1198.893204665249</v>
       </c>
       <c r="AK14" s="35" t="n">
-        <v>-5.516365380756992</v>
+        <v>-284.0375424669764</v>
       </c>
       <c r="AL14" s="39" t="n">
         <v>0.0423728813559322</v>
@@ -3626,13 +3973,38 @@
         </is>
       </c>
       <c r="AW14" s="37" t="n">
-        <v>57.09999672369963</v>
+        <v>56.94999750143358</v>
       </c>
       <c r="AX14" s="38" t="n">
-        <v>0.1</v>
+        <v>25</v>
       </c>
       <c r="AY14" s="38" t="n">
-        <v>12.37418739423011</v>
+        <v>21.05168050334063</v>
+      </c>
+      <c r="BA14" t="n">
+        <v>0.33</v>
+      </c>
+      <c r="BC14" t="n">
+        <v>80.84636</v>
+      </c>
+      <c r="BE14" t="n">
+        <v>100</v>
+      </c>
+      <c r="BF14" t="n">
+        <v>100</v>
+      </c>
+      <c r="BG14" t="n">
+        <v>100</v>
+      </c>
+      <c r="BI14" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="BJ14" t="inlineStr">
+        <is>
+          <t>Avoid</t>
+        </is>
       </c>
     </row>
     <row r="15" ht="15" customHeight="1" s="24">
@@ -3660,7 +4032,7 @@
         </is>
       </c>
       <c r="F15" s="32" t="n">
-        <v>1275407106048</v>
+        <v>1282227830784</v>
       </c>
       <c r="G15" s="32" t="inlineStr">
         <is>
@@ -3673,16 +4045,16 @@
         </is>
       </c>
       <c r="I15" s="32" t="n">
-        <v>27.5</v>
+        <v>62</v>
       </c>
       <c r="J15" s="32" t="n">
-        <v>22.1806031186621</v>
+        <v>17.2480260664295</v>
       </c>
       <c r="K15" s="32" t="n">
         <v>75</v>
       </c>
       <c r="L15" s="32" t="n">
-        <v>55</v>
+        <v>100</v>
       </c>
       <c r="M15" s="32" t="inlineStr">
         <is>
@@ -3709,7 +4081,7 @@
         <v>2.66</v>
       </c>
       <c r="S15" s="32" t="n">
-        <v>16.93883385059354</v>
+        <v>17.03115676692971</v>
       </c>
       <c r="T15" s="32" t="n">
         <v>0.1599527878445324</v>
@@ -3721,7 +4093,7 @@
         <v>0.1</v>
       </c>
       <c r="W15" s="32" t="n">
-        <v>0.04376054427538692</v>
+        <v>4.352332603335848</v>
       </c>
       <c r="X15" s="32" t="n">
         <v>8.460000000000001</v>
@@ -3760,22 +4132,22 @@
         </is>
       </c>
       <c r="AH15" s="33" t="n">
-        <v>696.1600644724707</v>
+        <v>663.0380119396805</v>
       </c>
       <c r="AI15" s="34" t="n">
         <v>1410</v>
       </c>
       <c r="AJ15" s="33" t="n">
-        <v>870.2000805905883</v>
+        <v>828.7975149246006</v>
       </c>
       <c r="AK15" s="35" t="n">
-        <v>-0.654562016384594</v>
+        <v>-74.65062019782788</v>
       </c>
       <c r="AL15" s="39" t="n">
-        <v>0.04661016949152542</v>
+        <v>2.414592883515921</v>
       </c>
       <c r="AM15" s="36" t="n">
-        <v>46610.16949152543</v>
+        <v>24145.92883515921</v>
       </c>
       <c r="AN15" s="32" t="inlineStr">
         <is>
@@ -3823,13 +4195,38 @@
         </is>
       </c>
       <c r="AW15" s="37" t="n">
-        <v>54.15000069201279</v>
+        <v>54.01000097311283</v>
       </c>
       <c r="AX15" s="38" t="n">
-        <v>0.1</v>
+        <v>5</v>
       </c>
       <c r="AY15" s="38" t="n">
-        <v>16.03168903077723</v>
+        <v>15.34526041334199</v>
+      </c>
+      <c r="BA15" t="n">
+        <v>3.63</v>
+      </c>
+      <c r="BC15" t="n">
+        <v>26.800592</v>
+      </c>
+      <c r="BE15" t="n">
+        <v>100</v>
+      </c>
+      <c r="BF15" t="n">
+        <v>44.3612062373242</v>
+      </c>
+      <c r="BG15" t="n">
+        <v>100</v>
+      </c>
+      <c r="BI15" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="BJ15" t="inlineStr">
+        <is>
+          <t>Avoid</t>
+        </is>
       </c>
     </row>
     <row r="16" ht="15" customHeight="1" s="24">
@@ -3857,7 +4254,7 @@
         </is>
       </c>
       <c r="F16" s="32" t="n">
-        <v>5486545469440</v>
+        <v>5491773145088</v>
       </c>
       <c r="G16" s="32" t="inlineStr">
         <is>
@@ -3870,16 +4267,16 @@
         </is>
       </c>
       <c r="I16" s="39" t="n">
-        <v>0</v>
+        <v>27</v>
       </c>
       <c r="J16" s="39" t="n">
-        <v>49.29197639221084</v>
+        <v>0.1911663741030732</v>
       </c>
       <c r="K16" s="32" t="n">
         <v>55</v>
       </c>
       <c r="L16" s="32" t="n">
-        <v>65</v>
+        <v>100</v>
       </c>
       <c r="M16" s="32" t="inlineStr">
         <is>
@@ -3906,7 +4303,7 @@
         <v>2.5</v>
       </c>
       <c r="S16" s="32" t="n">
-        <v>25.04568640202256</v>
+        <v>25.06499768969771</v>
       </c>
       <c r="T16" s="32" t="n">
         <v>0.1251375743928715</v>
@@ -3918,7 +4315,7 @@
         <v>1.12</v>
       </c>
       <c r="W16" s="32" t="n">
-        <v>0.01759846943853509</v>
+        <v>1.758491072569669</v>
       </c>
       <c r="X16" s="32" t="n">
         <v>12</v>
@@ -3957,24 +4354,22 @@
         </is>
       </c>
       <c r="AH16" s="33" t="n">
-        <v>1243.073274985581</v>
+        <v>1388.886139989236</v>
       </c>
       <c r="AI16" s="34" t="n">
         <v>3693</v>
       </c>
       <c r="AJ16" s="33" t="n">
-        <v>1553.841593731976</v>
+        <v>1736.107674986544</v>
       </c>
       <c r="AK16" s="35" t="n">
-        <v>-1.566606542190369</v>
-      </c>
-      <c r="AL16" s="39">
-        <f>IF(H16="Fail","Not Eligible (Failed Gate)",IF(J16="","Pending Score",IF(J16&gt;=90,"10%",IF(J16&gt;=80,"7.5%",IF(J16&gt;=70,"5%","Watchlist only")))))</f>
-        <v/>
-      </c>
-      <c r="AM16" s="36">
-        <f>IFERROR(ROUND(VALUE(SUBSTITUTE(AL16,"%",""))/100*Dashboard!$B$11,0),"")</f>
-        <v/>
+        <v>-129.9338950869472</v>
+      </c>
+      <c r="AL16" s="39" t="n">
+        <v>0.02676184304795499</v>
+      </c>
+      <c r="AM16" s="36" t="n">
+        <v>267.6184304795499</v>
       </c>
       <c r="AN16" s="32" t="inlineStr">
         <is>
@@ -4022,13 +4417,38 @@
         </is>
       </c>
       <c r="AW16" s="37" t="n">
-        <v>117.1900023096548</v>
+        <v>116.7799975894507</v>
       </c>
       <c r="AX16" s="38" t="n">
-        <v>0.1</v>
+        <v>12.0206624909</v>
       </c>
       <c r="AY16" s="38" t="n">
-        <v>13.28864785540046</v>
+        <v>14.86648120385806</v>
+      </c>
+      <c r="BA16" t="n">
+        <v>0.9399999999999999</v>
+      </c>
+      <c r="BC16" t="n">
+        <v>34.18308</v>
+      </c>
+      <c r="BE16" t="n">
+        <v>100</v>
+      </c>
+      <c r="BF16" t="n">
+        <v>98.58395278442168</v>
+      </c>
+      <c r="BG16" t="n">
+        <v>100</v>
+      </c>
+      <c r="BI16" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="BJ16" t="inlineStr">
+        <is>
+          <t>Avoid</t>
+        </is>
       </c>
     </row>
     <row r="17" ht="15" customHeight="1" s="24">
@@ -4056,7 +4476,7 @@
         </is>
       </c>
       <c r="F17" s="32" t="n">
-        <v>111188123648</v>
+        <v>109564600320</v>
       </c>
       <c r="G17" s="32" t="inlineStr">
         <is>
@@ -4069,16 +4489,16 @@
         </is>
       </c>
       <c r="I17" s="32" t="n">
-        <v>7</v>
+        <v>41</v>
       </c>
       <c r="J17" s="32" t="n">
-        <v>8.850832403821505</v>
+        <v>8.671158714433181</v>
       </c>
       <c r="K17" s="32" t="n">
         <v>70</v>
       </c>
       <c r="L17" s="32" t="n">
-        <v>40</v>
+        <v>100</v>
       </c>
       <c r="M17" s="32" t="inlineStr">
         <is>
@@ -4156,22 +4576,22 @@
         </is>
       </c>
       <c r="AH17" s="33" t="n">
-        <v/>
+        <v>86.62079174586319</v>
       </c>
       <c r="AI17" s="34" t="n">
         <v>1800</v>
       </c>
       <c r="AJ17" s="33" t="n">
-        <v/>
+        <v>108.275989682329</v>
       </c>
       <c r="AK17" s="35" t="n">
-        <v/>
+        <v>-1414.555539793545</v>
       </c>
       <c r="AL17" s="39" t="n">
-        <v>0.01186440677966102</v>
+        <v>1.213896479693902</v>
       </c>
       <c r="AM17" s="36" t="n">
-        <v>11864.40677966102</v>
+        <v>12138.96479693902</v>
       </c>
       <c r="AN17" s="32" t="inlineStr">
         <is>
@@ -4219,14 +4639,35 @@
         </is>
       </c>
       <c r="AW17" s="37" t="n">
-        <v>16.80999998030315</v>
+        <v>16.85000036990061</v>
       </c>
       <c r="AX17" s="38" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="AY17" s="38">
-        <f>IFERROR(IF(OR(T17="",T17=0,AW17="",T17-AX17&lt;3),"N/A",ROUND((1-(AX17/T17))*100/(Dashboard!$B$14-AX17),1)),"N/A")</f>
-        <v/>
+        <v>16.943</v>
+      </c>
+      <c r="AY17" s="38" t="n">
+        <v>6.425874758595191</v>
+      </c>
+      <c r="BC17" t="n">
+        <v>97.32344000000001</v>
+      </c>
+      <c r="BE17" t="n">
+        <v>100</v>
+      </c>
+      <c r="BF17" t="n">
+        <v>57.70166480764301</v>
+      </c>
+      <c r="BG17" t="n">
+        <v>100</v>
+      </c>
+      <c r="BI17" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="BJ17" t="inlineStr">
+        <is>
+          <t>Avoid</t>
+        </is>
       </c>
     </row>
     <row r="18" ht="15" customHeight="1" s="24">
@@ -4254,7 +4695,7 @@
         </is>
       </c>
       <c r="F18" s="32" t="n">
-        <v>1420631212032</v>
+        <v>1434018512896</v>
       </c>
       <c r="G18" s="32" t="inlineStr">
         <is>
@@ -4267,16 +4708,16 @@
         </is>
       </c>
       <c r="I18" s="32" t="n">
-        <v>10</v>
+        <v>40.5</v>
       </c>
       <c r="J18" s="32" t="n">
-        <v>20.43366572134297</v>
+        <v>11.9743653828561</v>
       </c>
       <c r="K18" s="32" t="n">
         <v>60</v>
       </c>
       <c r="L18" s="32" t="n">
-        <v>60</v>
+        <v>100</v>
       </c>
       <c r="M18" s="32" t="inlineStr">
         <is>
@@ -4303,7 +4744,7 @@
         <v>3.84</v>
       </c>
       <c r="S18" s="32" t="n">
-        <v>98.32949855953724</v>
+        <v>99.25580792648921</v>
       </c>
       <c r="T18" s="32" t="n">
         <v>0.1471374988564633</v>
@@ -4315,7 +4756,7 @@
         <v>0.1</v>
       </c>
       <c r="W18" s="32" t="n">
-        <v>-0.0005299462887530255</v>
+        <v>-0.05250005407760715</v>
       </c>
       <c r="X18" s="32" t="n">
         <v>25</v>
@@ -4354,22 +4795,22 @@
         </is>
       </c>
       <c r="AH18" s="33" t="n">
-        <v>34.75964440383766</v>
+        <v>32.95935151333484</v>
       </c>
       <c r="AI18" s="34" t="n">
         <v>965</v>
       </c>
       <c r="AJ18" s="33" t="n">
-        <v>43.44955550479708</v>
+        <v>41.19918939166855</v>
       </c>
       <c r="AK18" s="35" t="n">
-        <v>-19.75970604349253</v>
+        <v>-2109.99493787158</v>
       </c>
       <c r="AL18" s="39" t="n">
-        <v>0.01694915254237288</v>
+        <v>1.676320370035772</v>
       </c>
       <c r="AM18" s="36" t="n">
-        <v>16949.15254237288</v>
+        <v>16763.20370035772</v>
       </c>
       <c r="AN18" s="32" t="inlineStr">
         <is>
@@ -4417,13 +4858,38 @@
         </is>
       </c>
       <c r="AW18" s="37" t="n">
-        <v>7.960000204736147</v>
+        <v>7.679999838049428</v>
       </c>
       <c r="AX18" s="38" t="n">
-        <v>0.1</v>
+        <v>16.2591032</v>
       </c>
       <c r="AY18" s="38" t="n">
-        <v>5.628180764870088</v>
+        <v>5.36447778537351</v>
+      </c>
+      <c r="BA18" t="n">
+        <v>0.14</v>
+      </c>
+      <c r="BC18" t="n">
+        <v>118.55469</v>
+      </c>
+      <c r="BE18" t="n">
+        <v>100</v>
+      </c>
+      <c r="BF18" t="n">
+        <v>40.86733144268594</v>
+      </c>
+      <c r="BG18" t="n">
+        <v>100</v>
+      </c>
+      <c r="BI18" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="BJ18" t="inlineStr">
+        <is>
+          <t>Avoid</t>
+        </is>
       </c>
     </row>
     <row r="19" ht="15" customHeight="1" s="24">
@@ -4451,7 +4917,7 @@
         </is>
       </c>
       <c r="F19" s="32" t="n">
-        <v>98123816960</v>
+        <v>97146937344</v>
       </c>
       <c r="G19" s="32" t="inlineStr">
         <is>
@@ -4467,13 +4933,13 @@
         <v>0</v>
       </c>
       <c r="J19" s="32" t="n">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="K19" s="32" t="n">
         <v>70</v>
       </c>
       <c r="L19" s="32" t="n">
-        <v>30</v>
+        <v>90</v>
       </c>
       <c r="M19" s="32" t="inlineStr">
         <is>
@@ -4508,7 +4974,7 @@
         <v>0.9</v>
       </c>
       <c r="W19" s="32" t="n">
-        <v>-0.0539145798061806</v>
+        <v>-5.429653423358776</v>
       </c>
       <c r="X19" s="32" t="n">
         <v>-88</v>
@@ -4546,15 +5012,11 @@
           <t>Oct-2026</t>
         </is>
       </c>
-      <c r="AH19" s="33" t="n">
-        <v>-600.6663594578046</v>
-      </c>
+      <c r="AH19" s="33" t="n"/>
       <c r="AI19" s="34" t="n">
         <v>602</v>
       </c>
-      <c r="AJ19" s="33" t="n">
-        <v>-750.8329493222557</v>
-      </c>
+      <c r="AJ19" s="33" t="n"/>
       <c r="AK19" s="35" t="n">
         <v>1.735782840242523</v>
       </c>
@@ -4616,12 +5078,34 @@
         <v/>
       </c>
       <c r="AX19" s="38" t="n">
-        <v>0.1</v>
+        <v>5</v>
       </c>
       <c r="AY19" s="38">
         <f>IFERROR(IF(OR(T19="",T19=0,AW19="",T19-AX19&lt;3),"N/A",ROUND((1-(AX19/T19))*100/(Dashboard!$B$14-AX19),1)),"N/A")</f>
         <v/>
       </c>
+      <c r="BA19" t="n">
+        <v>0.42</v>
+      </c>
+      <c r="BE19" t="n">
+        <v>30</v>
+      </c>
+      <c r="BF19" t="n">
+        <v>100</v>
+      </c>
+      <c r="BG19" t="n">
+        <v>30</v>
+      </c>
+      <c r="BI19" t="inlineStr">
+        <is>
+          <t>Negative FCF / DCF Invalid | Missing EV/EBIT (EBIT &lt;= 0)</t>
+        </is>
+      </c>
+      <c r="BJ19" t="inlineStr">
+        <is>
+          <t>Avoid</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="15" customHeight="1" s="24">
       <c r="A20" s="32" t="n">
@@ -4648,7 +5132,7 @@
         </is>
       </c>
       <c r="F20" s="32" t="n">
-        <v>266978164736</v>
+        <v>259314909184</v>
       </c>
       <c r="G20" s="32" t="inlineStr">
         <is>
@@ -4661,16 +5145,16 @@
         </is>
       </c>
       <c r="I20" s="32" t="n">
+        <v>35</v>
+      </c>
+      <c r="J20" s="32" t="n">
         <v>0</v>
-      </c>
-      <c r="J20" s="32" t="n">
-        <v>30</v>
       </c>
       <c r="K20" s="32" t="n">
         <v>65</v>
       </c>
       <c r="L20" s="32" t="n">
-        <v>40</v>
+        <v>100</v>
       </c>
       <c r="M20" s="32" t="inlineStr">
         <is>
@@ -4697,7 +5181,7 @@
         <v>0.57</v>
       </c>
       <c r="S20" s="32" t="n">
-        <v>33.7754721391406</v>
+        <v>33.1920202449457</v>
       </c>
       <c r="T20" s="32" t="n">
         <v>0.09859652881090114</v>
@@ -4709,7 +5193,7 @@
         <v>0.65</v>
       </c>
       <c r="W20" s="32" t="n">
-        <v>-0.09180439231249965</v>
+        <v>-9.341813700760591</v>
       </c>
       <c r="X20" s="32" t="n">
         <v>42.3</v>
@@ -4747,15 +5231,11 @@
           <t>Oct-2026</t>
         </is>
       </c>
-      <c r="AH20" s="33" t="n">
-        <v>-427.7739838702832</v>
-      </c>
+      <c r="AH20" s="33" t="n"/>
       <c r="AI20" s="34" t="n">
         <v>270</v>
       </c>
-      <c r="AJ20" s="33" t="n">
-        <v>-534.7174798378539</v>
-      </c>
+      <c r="AJ20" s="33" t="n"/>
       <c r="AK20" s="35" t="n">
         <v>1.70691536045282</v>
       </c>
@@ -4816,10 +5296,35 @@
         <v>8.169999976224869</v>
       </c>
       <c r="AX20" s="38" t="n">
-        <v>0.1</v>
+        <v>9.896105979188</v>
       </c>
       <c r="AY20" s="38" t="n">
         <v>-64.8928980385745</v>
+      </c>
+      <c r="BA20" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="BC20" t="n">
+        <v>44.9388</v>
+      </c>
+      <c r="BE20" t="n">
+        <v>60</v>
+      </c>
+      <c r="BF20" t="n">
+        <v>100</v>
+      </c>
+      <c r="BG20" t="n">
+        <v>60</v>
+      </c>
+      <c r="BI20" t="inlineStr">
+        <is>
+          <t>Negative FCF / DCF Invalid</t>
+        </is>
+      </c>
+      <c r="BJ20" t="inlineStr">
+        <is>
+          <t>Avoid</t>
+        </is>
       </c>
     </row>
     <row r="21" ht="15" customHeight="1" s="24">
@@ -4847,7 +5352,7 @@
         </is>
       </c>
       <c r="F21" s="32" t="n">
-        <v>13646692352</v>
+        <v>13684156416</v>
       </c>
       <c r="G21" s="32" t="inlineStr">
         <is>
@@ -4860,16 +5365,16 @@
         </is>
       </c>
       <c r="I21" s="32" t="n">
-        <v>7</v>
+        <v>34</v>
       </c>
       <c r="J21" s="32" t="n">
-        <v>8.848264746087771</v>
+        <v>7.191589986330158</v>
       </c>
       <c r="K21" s="32" t="n">
         <v>70</v>
       </c>
       <c r="L21" s="32" t="n">
-        <v>35</v>
+        <v>100</v>
       </c>
       <c r="M21" s="32" t="inlineStr">
         <is>
@@ -4896,7 +5401,7 @@
         <v>5.08</v>
       </c>
       <c r="S21" s="32" t="n">
-        <v>22.74046380981408</v>
+        <v>22.79755625723865</v>
       </c>
       <c r="T21" s="32" t="n">
         <v>0.08622202272866382</v>
@@ -4908,7 +5413,7 @@
         <v>0.2</v>
       </c>
       <c r="W21" s="32" t="n">
-        <v>0.02443994470803409</v>
+        <v>2.437873918922504</v>
       </c>
       <c r="X21" s="32" t="n">
         <v>2</v>
@@ -4947,22 +5452,22 @@
         </is>
       </c>
       <c r="AH21" s="33" t="n">
-        <v/>
+        <v>204.8233857819562</v>
       </c>
       <c r="AI21" s="34" t="n">
         <v>495</v>
       </c>
       <c r="AJ21" s="33" t="n">
-        <v/>
+        <v>256.0292322274452</v>
       </c>
       <c r="AK21" s="35" t="n">
-        <v/>
+        <v>-92.59519536501655</v>
       </c>
       <c r="AL21" s="39" t="n">
-        <v>0.01186440677966102</v>
+        <v>1.006768075099032</v>
       </c>
       <c r="AM21" s="36" t="n">
-        <v>11864.40677966102</v>
+        <v>10067.68075099032</v>
       </c>
       <c r="AN21" s="32" t="inlineStr">
         <is>
@@ -5010,14 +5515,35 @@
         </is>
       </c>
       <c r="AW21" s="37" t="n">
-        <v>15.64999962128115</v>
+        <v>15.24999963661023</v>
       </c>
       <c r="AX21" s="38" t="n">
         <v>0.1</v>
       </c>
-      <c r="AY21" s="38">
-        <f>IFERROR(IF(OR(T21="",T21=0,AW21="",T21-AX21&lt;3),"N/A",ROUND((1-(AX21/T21))*100/(Dashboard!$B$14-AX21),1)),"N/A")</f>
-        <v/>
+      <c r="AY21" s="38" t="n">
+        <v>16.7888021132751</v>
+      </c>
+      <c r="BC21" t="n">
+        <v>32.334427</v>
+      </c>
+      <c r="BE21" t="n">
+        <v>100</v>
+      </c>
+      <c r="BF21" t="n">
+        <v>57.69652949217554</v>
+      </c>
+      <c r="BG21" t="n">
+        <v>100</v>
+      </c>
+      <c r="BI21" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="BJ21" t="inlineStr">
+        <is>
+          <t>Avoid</t>
+        </is>
       </c>
     </row>
     <row r="22" ht="15" customHeight="1" s="24">
@@ -5045,7 +5571,7 @@
         </is>
       </c>
       <c r="F22" s="32" t="n">
-        <v>46938255360</v>
+        <v>47008841728</v>
       </c>
       <c r="G22" s="32" t="inlineStr">
         <is>
@@ -5058,16 +5584,16 @@
         </is>
       </c>
       <c r="I22" s="39" t="n">
+        <v>10</v>
+      </c>
+      <c r="J22" s="39" t="n">
         <v>0</v>
-      </c>
-      <c r="J22" s="39" t="n">
-        <v>50</v>
       </c>
       <c r="K22" s="32" t="n">
         <v>45</v>
       </c>
       <c r="L22" s="32" t="n">
-        <v>35</v>
+        <v>100</v>
       </c>
       <c r="M22" s="32" t="inlineStr">
         <is>
@@ -5094,7 +5620,7 @@
         <v>6.97</v>
       </c>
       <c r="S22" s="32" t="n">
-        <v>42.65630599301274</v>
+        <v>42.69175778834506</v>
       </c>
       <c r="T22" s="32" t="n">
         <v>0.08870267856766871</v>
@@ -5106,7 +5632,7 @@
         <v>1.2</v>
       </c>
       <c r="W22" s="32" t="n">
-        <v>0.01296823296423419</v>
+        <v>1.295746397357447</v>
       </c>
       <c r="X22" s="32" t="n">
         <v>7.5</v>
@@ -5145,16 +5671,16 @@
         </is>
       </c>
       <c r="AH22" s="33" t="n">
-        <v>60.74983976802167</v>
+        <v>64.30133761446289</v>
       </c>
       <c r="AI22" s="34" t="n">
         <v>230</v>
       </c>
       <c r="AJ22" s="33" t="n">
-        <v>75.93729971002708</v>
+        <v>80.37667201807862</v>
       </c>
       <c r="AK22" s="35" t="n">
-        <v>-2.064896972749059</v>
+        <v>-189.9970776938519</v>
       </c>
       <c r="AL22" s="39">
         <f>IF(H22="Fail","Not Eligible (Failed Gate)",IF(J22="","Pending Score",IF(J22&gt;=90,"10%",IF(J22&gt;=80,"7.5%",IF(J22&gt;=70,"5%","Watchlist only")))))</f>
@@ -5210,13 +5736,35 @@
         </is>
       </c>
       <c r="AW22" s="37" t="n">
-        <v>3.430000121584176</v>
+        <v>3.440000047226394</v>
       </c>
       <c r="AX22" s="38" t="n">
-        <v>0.1</v>
+        <v>8.972</v>
       </c>
       <c r="AY22" s="38" t="n">
-        <v>22.01081151015277</v>
+        <v>23.36531163316239</v>
+      </c>
+      <c r="BC22" t="n">
+        <v>67.75872</v>
+      </c>
+      <c r="BE22" t="n">
+        <v>100</v>
+      </c>
+      <c r="BF22" t="n">
+        <v>100</v>
+      </c>
+      <c r="BG22" t="n">
+        <v>100</v>
+      </c>
+      <c r="BI22" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="BJ22" t="inlineStr">
+        <is>
+          <t>Avoid</t>
+        </is>
       </c>
     </row>
     <row r="23" ht="15" customHeight="1" s="24">
@@ -5244,7 +5792,7 @@
         </is>
       </c>
       <c r="F23" s="32" t="n">
-        <v>1373667328000</v>
+        <v>1363437027328</v>
       </c>
       <c r="G23" s="32" t="inlineStr">
         <is>
@@ -5257,16 +5805,16 @@
         </is>
       </c>
       <c r="I23" s="39" t="n">
+        <v>33.33333333333334</v>
+      </c>
+      <c r="J23" s="39" t="n">
         <v>0</v>
-      </c>
-      <c r="J23" s="39" t="n">
-        <v>50</v>
       </c>
       <c r="K23" s="32" t="n">
         <v>50</v>
       </c>
       <c r="L23" s="32" t="n">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="M23" s="32" t="inlineStr">
         <is>
@@ -5303,7 +5851,7 @@
         <v>8.25</v>
       </c>
       <c r="W23" s="32" t="n">
-        <v>-0.004083075974278943</v>
+        <v>-0.408660169143568</v>
       </c>
       <c r="X23" s="32" t="n">
         <v>10</v>
@@ -5342,16 +5890,16 @@
         </is>
       </c>
       <c r="AH23" s="33" t="n">
-        <v>281.2038884702938</v>
+        <v>233.4636678160078</v>
       </c>
       <c r="AI23" s="34" t="n">
         <v>423</v>
       </c>
       <c r="AJ23" s="33" t="n">
-        <v>351.5048605878673</v>
+        <v>291.8295847700098</v>
       </c>
       <c r="AK23" s="35" t="n">
-        <v>-0.1841941511245422</v>
+        <v>-41.57234960451407</v>
       </c>
       <c r="AL23" s="39">
         <f>IF(H23="Fail","Not Eligible (Failed Gate)",IF(J23="","Pending Score",IF(J23&gt;=90,"10%",IF(J23&gt;=80,"7.5%",IF(J23&gt;=70,"5%","Watchlist only")))))</f>
@@ -5407,13 +5955,38 @@
         </is>
       </c>
       <c r="AW23" s="37" t="n">
-        <v>78.46999995287088</v>
+        <v>78.48999796342059</v>
       </c>
       <c r="AX23" s="38" t="n">
-        <v>0.1</v>
+        <v>16.12516180932</v>
       </c>
       <c r="AY23" s="38" t="n">
-        <v>4.478339413783504</v>
+        <v>3.718047964963815</v>
+      </c>
+      <c r="BA23" t="n">
+        <v>3.75</v>
+      </c>
+      <c r="BC23" t="n">
+        <v>5.263728</v>
+      </c>
+      <c r="BE23" t="n">
+        <v>60</v>
+      </c>
+      <c r="BF23" t="n">
+        <v>100</v>
+      </c>
+      <c r="BG23" t="n">
+        <v>100</v>
+      </c>
+      <c r="BI23" t="inlineStr">
+        <is>
+          <t>Missing EV/EBIT (EBIT &lt;= 0)</t>
+        </is>
+      </c>
+      <c r="BJ23" t="inlineStr">
+        <is>
+          <t>Avoid</t>
+        </is>
       </c>
     </row>
     <row r="24" ht="15" customHeight="1" s="24">
@@ -5441,7 +6014,7 @@
         </is>
       </c>
       <c r="F24" s="32" t="n">
-        <v>3613498540032</v>
+        <v>3617883947008</v>
       </c>
       <c r="G24" s="32" t="inlineStr">
         <is>
@@ -5454,16 +6027,16 @@
         </is>
       </c>
       <c r="I24" s="39" t="n">
-        <v>35</v>
+        <v>77</v>
       </c>
       <c r="J24" s="39" t="n">
-        <v>20.98775651125753</v>
+        <v>22.3394274863317</v>
       </c>
       <c r="K24" s="32" t="n">
         <v>80</v>
       </c>
       <c r="L24" s="32" t="n">
-        <v>80</v>
+        <v>100</v>
       </c>
       <c r="M24" s="32" t="inlineStr">
         <is>
@@ -5490,7 +6063,7 @@
         <v>2.71</v>
       </c>
       <c r="S24" s="32" t="n">
-        <v>14.20057846027863</v>
+        <v>14.21771194125227</v>
       </c>
       <c r="T24" s="32" t="n">
         <v>0.2839112472627043</v>
@@ -5502,7 +6075,7 @@
         <v>0.03</v>
       </c>
       <c r="W24" s="32" t="n">
-        <v>0.04479421678042514</v>
+        <v>4.474023616356444</v>
       </c>
       <c r="X24" s="32" t="n">
         <v>9.869999999999999</v>
@@ -5541,22 +6114,22 @@
         </is>
       </c>
       <c r="AH24" s="33" t="n">
-        <v>151.1265579438416</v>
+        <v>143.9580476888378</v>
       </c>
       <c r="AI24" s="34" t="n">
         <v>289</v>
       </c>
       <c r="AJ24" s="33" t="n">
-        <v>188.9081974298019</v>
+        <v>179.9475596110472</v>
       </c>
       <c r="AK24" s="35" t="n">
-        <v>-0.5266674708871175</v>
+        <v>-60.4634153550773</v>
       </c>
       <c r="AL24" s="39" t="n">
-        <v>0.05932203389830508</v>
+        <v>3.127350481879385</v>
       </c>
       <c r="AM24" s="36" t="n">
-        <v>59322.03389830508</v>
+        <v>31273.50481879385</v>
       </c>
       <c r="AN24" s="32" t="inlineStr">
         <is>
@@ -5607,10 +6180,35 @@
         <v>16.40000079611654</v>
       </c>
       <c r="AX24" s="38" t="n">
-        <v>0.1</v>
+        <v>5</v>
       </c>
       <c r="AY24" s="38" t="n">
-        <v>11.43512090979431</v>
+        <v>10.97241217140532</v>
+      </c>
+      <c r="BA24" t="n">
+        <v>5.55</v>
+      </c>
+      <c r="BC24" t="n">
+        <v>17.606709</v>
+      </c>
+      <c r="BE24" t="n">
+        <v>100</v>
+      </c>
+      <c r="BF24" t="n">
+        <v>41.97551302251505</v>
+      </c>
+      <c r="BG24" t="n">
+        <v>100</v>
+      </c>
+      <c r="BI24" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="BJ24" t="inlineStr">
+        <is>
+          <t>Avoid</t>
+        </is>
       </c>
     </row>
     <row r="25" ht="15" customHeight="1" s="24">
@@ -5638,7 +6236,7 @@
         </is>
       </c>
       <c r="F25" s="32" t="n">
-        <v>2075201372160</v>
+        <v>2068613431296</v>
       </c>
       <c r="G25" s="32" t="inlineStr">
         <is>
@@ -5651,16 +6249,16 @@
         </is>
       </c>
       <c r="I25" s="39" t="n">
-        <v>10</v>
+        <v>72</v>
       </c>
       <c r="J25" s="39" t="n">
-        <v>0.6142791975346761</v>
+        <v>21.15771897777503</v>
       </c>
       <c r="K25" s="32" t="n">
         <v>80</v>
       </c>
       <c r="L25" s="32" t="n">
-        <v>75</v>
+        <v>100</v>
       </c>
       <c r="M25" s="32" t="inlineStr">
         <is>
@@ -5687,7 +6285,7 @@
         <v>1.95</v>
       </c>
       <c r="S25" s="32" t="n">
-        <v>42.02475321374401</v>
+        <v>41.89152084648209</v>
       </c>
       <c r="T25" s="32" t="n">
         <v>0.2197289657631528</v>
@@ -5699,7 +6297,7 @@
         <v>0.05</v>
       </c>
       <c r="W25" s="32" t="n">
-        <v>0.01698548337047286</v>
+        <v>1.703950423466705</v>
       </c>
       <c r="X25" s="32" t="n">
         <v>15.6</v>
@@ -5738,22 +6336,22 @@
         </is>
       </c>
       <c r="AH25" s="33" t="n">
-        <v/>
+        <v>2111.405238040509</v>
       </c>
       <c r="AI25" s="34" t="n">
         <v>7454</v>
       </c>
       <c r="AJ25" s="33" t="n">
-        <v/>
+        <v>2639.256547550636</v>
       </c>
       <c r="AK25" s="35" t="n">
-        <v/>
+        <v>-185.5349551749257</v>
       </c>
       <c r="AL25" s="39" t="n">
-        <v>0.01694915254237288</v>
+        <v>2.961920249795917</v>
       </c>
       <c r="AM25" s="36" t="n">
-        <v>16949.15254237288</v>
+        <v>29619.20249795917</v>
       </c>
       <c r="AN25" s="32" t="inlineStr">
         <is>
@@ -5801,14 +6399,38 @@
         </is>
       </c>
       <c r="AW25" s="37" t="n">
-        <v>200.3699953883096</v>
+        <v>200.9799908097525</v>
       </c>
       <c r="AX25" s="38" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="AY25" s="38">
-        <f>IFERROR(IF(OR(T25="",T25=0,AW25="",T25-AX25&lt;3),"N/A",ROUND((1-(AX25/T25))*100/(Dashboard!$B$14-AX25),1)),"N/A")</f>
-        <v/>
+        <v>15.4840062</v>
+      </c>
+      <c r="AY25" s="38" t="n">
+        <v>13.13193625012756</v>
+      </c>
+      <c r="BA25" t="n">
+        <v>0.9399999999999999</v>
+      </c>
+      <c r="BC25" t="n">
+        <v>37.49627</v>
+      </c>
+      <c r="BE25" t="n">
+        <v>100</v>
+      </c>
+      <c r="BF25" t="n">
+        <v>41.22855839506935</v>
+      </c>
+      <c r="BG25" t="n">
+        <v>100</v>
+      </c>
+      <c r="BI25" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="BJ25" t="inlineStr">
+        <is>
+          <t>Avoid</t>
+        </is>
       </c>
     </row>
     <row r="26" ht="15" customHeight="1" s="24">
@@ -5836,7 +6458,7 @@
         </is>
       </c>
       <c r="F26" s="32" t="n">
-        <v>252500983808</v>
+        <v>253462151168</v>
       </c>
       <c r="G26" s="32" t="inlineStr">
         <is>
@@ -5849,16 +6471,16 @@
         </is>
       </c>
       <c r="I26" s="39" t="n">
+        <v>35</v>
+      </c>
+      <c r="J26" s="39" t="n">
         <v>0</v>
-      </c>
-      <c r="J26" s="39" t="n">
-        <v>30</v>
       </c>
       <c r="K26" s="32" t="n">
         <v>55</v>
       </c>
       <c r="L26" s="32" t="n">
-        <v>50</v>
+        <v>100</v>
       </c>
       <c r="M26" s="32" t="inlineStr">
         <is>
@@ -5935,18 +6557,12 @@
           <t>Sep-2026</t>
         </is>
       </c>
-      <c r="AH26" s="33" t="n">
-        <v/>
-      </c>
+      <c r="AH26" s="33" t="n"/>
       <c r="AI26" s="34" t="n">
         <v>1460</v>
       </c>
-      <c r="AJ26" s="33" t="n">
-        <v/>
-      </c>
-      <c r="AK26" s="35" t="n">
-        <v/>
-      </c>
+      <c r="AJ26" s="33" t="n"/>
+      <c r="AK26" s="35" t="n"/>
       <c r="AL26" s="39">
         <f>IF(H26="Fail","Not Eligible (Failed Gate)",IF(J26="","Pending Score",IF(J26&gt;=90,"10%",IF(J26&gt;=80,"7.5%",IF(J26&gt;=70,"5%","Watchlist only")))))</f>
         <v/>
@@ -6001,15 +6617,37 @@
         </is>
       </c>
       <c r="AW26" s="37" t="n">
-        <v>48.44000116413351</v>
+        <v>48.40999983783782</v>
       </c>
       <c r="AX26" s="38" t="n">
-        <v>0.1</v>
+        <v>10.5100006</v>
       </c>
       <c r="AY26" s="38">
         <f>IFERROR(IF(OR(T26="",T26=0,AW26="",T26-AX26&lt;3),"N/A",ROUND((1-(AX26/T26))*100/(Dashboard!$B$14-AX26),1)),"N/A")</f>
         <v/>
       </c>
+      <c r="BC26" t="n">
+        <v>32.68333</v>
+      </c>
+      <c r="BE26" t="n">
+        <v>60</v>
+      </c>
+      <c r="BF26" t="n">
+        <v>100</v>
+      </c>
+      <c r="BG26" t="n">
+        <v>60</v>
+      </c>
+      <c r="BI26" t="inlineStr">
+        <is>
+          <t>Negative FCF / DCF Invalid</t>
+        </is>
+      </c>
+      <c r="BJ26" t="inlineStr">
+        <is>
+          <t>Avoid</t>
+        </is>
+      </c>
     </row>
     <row r="27" ht="15" customHeight="1" s="24">
       <c r="A27" s="32" t="n">
@@ -6036,7 +6674,7 @@
         </is>
       </c>
       <c r="F27" s="32" t="n">
-        <v>1192392785920</v>
+        <v>1192852586496</v>
       </c>
       <c r="G27" s="32" t="inlineStr">
         <is>
@@ -6049,16 +6687,16 @@
         </is>
       </c>
       <c r="I27" s="32" t="n">
-        <v>0</v>
+        <v>16.66666666666667</v>
       </c>
       <c r="J27" s="32" t="n">
-        <v>17.17786299442293</v>
+        <v>18.39276571773325</v>
       </c>
       <c r="K27" s="32" t="n">
         <v>70</v>
       </c>
       <c r="L27" s="32" t="n">
-        <v>50</v>
+        <v>60</v>
       </c>
       <c r="M27" s="32" t="inlineStr">
         <is>
@@ -6095,7 +6733,7 @@
         <v>0.66</v>
       </c>
       <c r="W27" s="32" t="n">
-        <v>0.5706665849911694</v>
+        <v>57.0043635432243</v>
       </c>
       <c r="X27" s="32" t="n">
         <v>9.800000000000001</v>
@@ -6134,24 +6772,22 @@
         </is>
       </c>
       <c r="AH27" s="33" t="n">
-        <v/>
+        <v>260.3949652129983</v>
       </c>
       <c r="AI27" s="34" t="n">
         <v>106</v>
       </c>
       <c r="AJ27" s="33" t="n">
-        <v/>
+        <v>325.4937065162478</v>
       </c>
       <c r="AK27" s="35" t="n">
-        <v/>
-      </c>
-      <c r="AL27" s="39">
-        <f>IF(H27="Fail","Not Eligible (Failed Gate)",IF(J27="","Pending Score",IF(J27&gt;=90,"10%",IF(J27&gt;=80,"7.5%",IF(J27&gt;=70,"5%","Watchlist only")))))</f>
-        <v/>
-      </c>
-      <c r="AM27" s="36">
-        <f>IFERROR(ROUND(VALUE(SUBSTITUTE(AL27,"%",""))/100*Dashboard!$B$11,0),"")</f>
-        <v/>
+        <v>68.11305474663023</v>
+      </c>
+      <c r="AL27" s="39" t="n">
+        <v>1.544908653517862</v>
+      </c>
+      <c r="AM27" s="36" t="n">
+        <v>15449.08653517863</v>
       </c>
       <c r="AN27" s="32" t="inlineStr">
         <is>
@@ -6199,14 +6835,38 @@
         </is>
       </c>
       <c r="AW27" s="37" t="n">
-        <v>15.83999936487328</v>
+        <v>16</v>
       </c>
       <c r="AX27" s="38" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="AY27" s="38">
-        <f>IFERROR(IF(OR(T27="",T27=0,AW27="",T27-AX27&lt;3),"N/A",ROUND((1-(AX27/T27))*100/(Dashboard!$B$14-AX27),1)),"N/A")</f>
-        <v/>
+        <v>10.6308197597</v>
+      </c>
+      <c r="AY27" s="38" t="n">
+        <v>20.34335665726549</v>
+      </c>
+      <c r="BA27" t="n">
+        <v>2.88</v>
+      </c>
+      <c r="BC27" t="n">
+        <v>6.486875</v>
+      </c>
+      <c r="BE27" t="n">
+        <v>60</v>
+      </c>
+      <c r="BF27" t="n">
+        <v>34.35572598884587</v>
+      </c>
+      <c r="BG27" t="n">
+        <v>100</v>
+      </c>
+      <c r="BI27" t="inlineStr">
+        <is>
+          <t>Missing EV/EBIT (EBIT &lt;= 0)</t>
+        </is>
+      </c>
+      <c r="BJ27" t="inlineStr">
+        <is>
+          <t>Avoid</t>
+        </is>
       </c>
     </row>
     <row r="28" ht="15" customHeight="1" s="24">
@@ -6234,7 +6894,7 @@
         </is>
       </c>
       <c r="F28" s="32" t="n">
-        <v>664257560576</v>
+        <v>671207784448</v>
       </c>
       <c r="G28" s="32" t="inlineStr">
         <is>
@@ -6247,16 +6907,16 @@
         </is>
       </c>
       <c r="I28" s="39" t="n">
-        <v>27.5</v>
+        <v>79</v>
       </c>
       <c r="J28" s="39" t="n">
-        <v>22.2554387124765</v>
+        <v>21.91820341714357</v>
       </c>
       <c r="K28" s="32" t="n">
         <v>93</v>
       </c>
       <c r="L28" s="32" t="n">
-        <v>73</v>
+        <v>100</v>
       </c>
       <c r="M28" s="32" t="inlineStr">
         <is>
@@ -6283,7 +6943,7 @@
         <v>0.4</v>
       </c>
       <c r="S28" s="32" t="n">
-        <v>27.99871264859378</v>
+        <v>28.29265318029181</v>
       </c>
       <c r="T28" s="32" t="n">
         <v>0.160702848996963</v>
@@ -6295,7 +6955,7 @@
         <v>0.7</v>
       </c>
       <c r="W28" s="32" t="n">
-        <v>0.01584823492001085</v>
+        <v>1.568358303780037</v>
       </c>
       <c r="X28" s="32" t="n">
         <v>35.9</v>
@@ -6334,22 +6994,22 @@
         </is>
       </c>
       <c r="AH28" s="33" t="n">
-        <v>442.1754954230594</v>
+        <v>393.9612520419522</v>
       </c>
       <c r="AI28" s="34" t="n">
         <v>1464</v>
       </c>
       <c r="AJ28" s="33" t="n">
-        <v>552.7193692788242</v>
+        <v>492.4515650524402</v>
       </c>
       <c r="AK28" s="35" t="n">
-        <v>-1.714759213084605</v>
+        <v>-207.8881473020687</v>
       </c>
       <c r="AL28" s="39" t="n">
-        <v>0.04661016949152542</v>
+        <v>3.068382305700264</v>
       </c>
       <c r="AM28" s="36" t="n">
-        <v>46610.16949152543</v>
+        <v>30683.82305700264</v>
       </c>
       <c r="AN28" s="32" t="inlineStr">
         <is>
@@ -6400,10 +7060,35 @@
         <v>44.31000216574179</v>
       </c>
       <c r="AX28" s="38" t="n">
-        <v>0.1</v>
+        <v>11.89214301142002</v>
       </c>
       <c r="AY28" s="38" t="n">
-        <v>11.90179520410905</v>
+        <v>11.11377939635388</v>
+      </c>
+      <c r="BA28" t="n">
+        <v>1.08</v>
+      </c>
+      <c r="BC28" t="n">
+        <v>34.218006</v>
+      </c>
+      <c r="BE28" t="n">
+        <v>100</v>
+      </c>
+      <c r="BF28" t="n">
+        <v>44.510877424953</v>
+      </c>
+      <c r="BG28" t="n">
+        <v>100</v>
+      </c>
+      <c r="BI28" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="BJ28" t="inlineStr">
+        <is>
+          <t>Avoid</t>
+        </is>
       </c>
     </row>
     <row r="29" ht="15" customHeight="1" s="24">
@@ -6431,7 +7116,7 @@
         </is>
       </c>
       <c r="F29" s="32" t="n">
-        <v>466008768512</v>
+        <v>462353268736</v>
       </c>
       <c r="G29" s="32" t="inlineStr">
         <is>
@@ -6444,16 +7129,16 @@
         </is>
       </c>
       <c r="I29" s="39" t="n">
-        <v>17.5</v>
+        <v>72.5</v>
       </c>
       <c r="J29" s="39" t="n">
-        <v>25.80162640632039</v>
+        <v>10.14606951805904</v>
       </c>
       <c r="K29" s="32" t="n">
         <v>80</v>
       </c>
       <c r="L29" s="32" t="n">
-        <v>72</v>
+        <v>100</v>
       </c>
       <c r="M29" s="32" t="inlineStr">
         <is>
@@ -6480,7 +7165,7 @@
         <v>0.5</v>
       </c>
       <c r="S29" s="32" t="n">
-        <v>25.37712846688706</v>
+        <v>25.18720583478938</v>
       </c>
       <c r="T29" s="32" t="n">
         <v>0.3502647805451143</v>
@@ -6492,7 +7177,7 @@
         <v>0.86</v>
       </c>
       <c r="W29" s="32" t="n">
-        <v>-0.03555566321685065</v>
+        <v>-3.582376858703013</v>
       </c>
       <c r="X29" s="32" t="n">
         <v>44</v>
@@ -6530,23 +7215,19 @@
           <t>Oct-2026</t>
         </is>
       </c>
-      <c r="AH29" s="33" t="n">
-        <v>-166.8453885131904</v>
-      </c>
+      <c r="AH29" s="33" t="n"/>
       <c r="AI29" s="34" t="n">
         <v>1065</v>
       </c>
-      <c r="AJ29" s="33" t="n">
-        <v>-208.5567356414879</v>
-      </c>
+      <c r="AJ29" s="33" t="n"/>
       <c r="AK29" s="35" t="n">
         <v>5.95117070577406</v>
       </c>
       <c r="AL29" s="39" t="n">
-        <v>0.02966101694915254</v>
+        <v>0.8522236861055931</v>
       </c>
       <c r="AM29" s="36" t="n">
-        <v>29661.01694915254</v>
+        <v>8522.23686105593</v>
       </c>
       <c r="AN29" s="32" t="inlineStr">
         <is>
@@ -6597,10 +7278,35 @@
         <v>32.84000078744762</v>
       </c>
       <c r="AX29" s="38" t="n">
-        <v>0.1</v>
+        <v>25</v>
       </c>
       <c r="AY29" s="38" t="n">
         <v>-6.201508642327919</v>
+      </c>
+      <c r="BA29" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="BC29" t="n">
+        <v>31.19671</v>
+      </c>
+      <c r="BE29" t="n">
+        <v>60</v>
+      </c>
+      <c r="BF29" t="n">
+        <v>86.00542135440132</v>
+      </c>
+      <c r="BG29" t="n">
+        <v>60</v>
+      </c>
+      <c r="BI29" t="inlineStr">
+        <is>
+          <t>Negative FCF / DCF Invalid</t>
+        </is>
+      </c>
+      <c r="BJ29" t="inlineStr">
+        <is>
+          <t>Avoid</t>
+        </is>
       </c>
     </row>
     <row r="30" ht="15" customHeight="1" s="24">
@@ -6628,7 +7334,7 @@
         </is>
       </c>
       <c r="F30" s="32" t="n">
-        <v>344627937280</v>
+        <v>347010990080</v>
       </c>
       <c r="G30" s="32" t="inlineStr">
         <is>
@@ -6641,16 +7347,16 @@
         </is>
       </c>
       <c r="I30" s="39" t="n">
-        <v>10</v>
+        <v>56.66666666666667</v>
       </c>
       <c r="J30" s="39" t="n">
-        <v>21.86724794139225</v>
+        <v>15.94189283321106</v>
       </c>
       <c r="K30" s="32" t="n">
         <v>92</v>
       </c>
       <c r="L30" s="32" t="n">
-        <v>79</v>
+        <v>60</v>
       </c>
       <c r="M30" s="32" t="inlineStr">
         <is>
@@ -6687,7 +7393,7 @@
         <v>0.05</v>
       </c>
       <c r="W30" s="32" t="n">
-        <v>0.05360916928054234</v>
+        <v>5.323038836525122</v>
       </c>
       <c r="X30" s="32" t="n">
         <v>26.4</v>
@@ -6726,22 +7432,22 @@
         </is>
       </c>
       <c r="AH30" s="33" t="n">
-        <v>282.8861590541263</v>
+        <v>313.1083018493239</v>
       </c>
       <c r="AI30" s="34" t="n">
         <v>587</v>
       </c>
       <c r="AJ30" s="33" t="n">
-        <v>353.6076988176578</v>
+        <v>391.3853773116548</v>
       </c>
       <c r="AK30" s="35" t="n">
-        <v>-0.6563553394294831</v>
+        <v>-50.68268621859886</v>
       </c>
       <c r="AL30" s="39" t="n">
-        <v>0.01694915254237288</v>
+        <v>1.33904647998297</v>
       </c>
       <c r="AM30" s="36" t="n">
-        <v>16949.15254237288</v>
+        <v>13390.4647998297</v>
       </c>
       <c r="AN30" s="32" t="inlineStr">
         <is>
@@ -6789,13 +7495,35 @@
         </is>
       </c>
       <c r="AW30" s="37" t="n">
-        <v>9.459999883708386</v>
+        <v>9.47999933129636</v>
       </c>
       <c r="AX30" s="38" t="n">
         <v>0.1</v>
       </c>
       <c r="AY30" s="38" t="n">
-        <v>37.33977812224475</v>
+        <v>41.28537735355008</v>
+      </c>
+      <c r="BC30" t="n">
+        <v>62.20992</v>
+      </c>
+      <c r="BE30" t="n">
+        <v>60</v>
+      </c>
+      <c r="BF30" t="n">
+        <v>43.7344958827845</v>
+      </c>
+      <c r="BG30" t="n">
+        <v>100</v>
+      </c>
+      <c r="BI30" t="inlineStr">
+        <is>
+          <t>Missing EV/EBIT (EBIT &lt;= 0)</t>
+        </is>
+      </c>
+      <c r="BJ30" t="inlineStr">
+        <is>
+          <t>Avoid</t>
+        </is>
       </c>
     </row>
     <row r="31" ht="15" customHeight="1" s="24">
@@ -6823,7 +7551,7 @@
         </is>
       </c>
       <c r="F31" s="32" t="n">
-        <v>65705717760</v>
+        <v>66477535232</v>
       </c>
       <c r="G31" s="32" t="inlineStr">
         <is>
@@ -6836,16 +7564,16 @@
         </is>
       </c>
       <c r="I31" s="39" t="n">
-        <v>24.5</v>
+        <v>55</v>
       </c>
       <c r="J31" s="39" t="n">
-        <v>6.109657928630957</v>
+        <v>13.13968813925297</v>
       </c>
       <c r="K31" s="32" t="n">
         <v>40</v>
       </c>
       <c r="L31" s="32" t="n">
-        <v>30</v>
+        <v>100</v>
       </c>
       <c r="M31" s="32" t="inlineStr">
         <is>
@@ -6872,7 +7600,7 @@
         <v>0.07000000000000001</v>
       </c>
       <c r="S31" s="32" t="n">
-        <v>9.514755669816196</v>
+        <v>9.617035983090602</v>
       </c>
       <c r="T31" s="32" t="n">
         <v>0.1485027274793545</v>
@@ -6884,7 +7612,7 @@
         <v>1.81</v>
       </c>
       <c r="W31" s="32" t="n">
-        <v>-0.01288940183082927</v>
+        <v>-1.275231883982301</v>
       </c>
       <c r="X31" s="32" t="n">
         <v>28.5</v>
@@ -6923,22 +7651,22 @@
         </is>
       </c>
       <c r="AH31" s="33" t="n">
-        <v/>
+        <v>32.55699896453103</v>
       </c>
       <c r="AI31" s="34" t="n">
         <v>189</v>
       </c>
       <c r="AJ31" s="33" t="n">
-        <v/>
+        <v>40.69624870566378</v>
       </c>
       <c r="AK31" s="35" t="n">
-        <v/>
+        <v>-350.8032210213702</v>
       </c>
       <c r="AL31" s="39" t="n">
-        <v>0.04152542372881356</v>
+        <v>1.83945672104533</v>
       </c>
       <c r="AM31" s="36" t="n">
-        <v>41525.42372881356</v>
+        <v>18394.5672104533</v>
       </c>
       <c r="AN31" s="32" t="inlineStr">
         <is>
@@ -6989,11 +7717,32 @@
         <v>13.39000066089729</v>
       </c>
       <c r="AX31" s="38" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="AY31" s="38">
-        <f>IFERROR(IF(OR(T31="",T31=0,AW31="",T31-AX31&lt;3),"N/A",ROUND((1-(AX31/T31))*100/(Dashboard!$B$14-AX31),1)),"N/A")</f>
-        <v/>
+        <v>21.336001</v>
+      </c>
+      <c r="AY31" s="38" t="n">
+        <v>3.039301621035383</v>
+      </c>
+      <c r="BC31" t="n">
+        <v>13.70127</v>
+      </c>
+      <c r="BE31" t="n">
+        <v>100</v>
+      </c>
+      <c r="BF31" t="n">
+        <v>52.21931585726192</v>
+      </c>
+      <c r="BG31" t="n">
+        <v>100</v>
+      </c>
+      <c r="BI31" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="BJ31" t="inlineStr">
+        <is>
+          <t>Avoid</t>
+        </is>
       </c>
     </row>
     <row r="32" ht="15" customHeight="1" s="24">
@@ -7021,7 +7770,7 @@
         </is>
       </c>
       <c r="F32" s="32" t="n">
-        <v>100332027904</v>
+        <v>99282051072</v>
       </c>
       <c r="G32" s="32" t="inlineStr">
         <is>
@@ -7034,16 +7783,16 @@
         </is>
       </c>
       <c r="I32" s="32" t="n">
-        <v>24.5</v>
+        <v>85</v>
       </c>
       <c r="J32" s="32" t="n">
-        <v>9.169029203710329</v>
+        <v>100</v>
       </c>
       <c r="K32" s="32" t="n">
         <v>70</v>
       </c>
       <c r="L32" s="32" t="n">
-        <v>60</v>
+        <v>100</v>
       </c>
       <c r="M32" s="32" t="inlineStr">
         <is>
@@ -7070,7 +7819,7 @@
         <v>0.3</v>
       </c>
       <c r="S32" s="32" t="n">
-        <v>11.02401450768475</v>
+        <v>10.91874628515284</v>
       </c>
       <c r="T32" s="32" t="n">
         <v>0.2008202361619554</v>
@@ -7082,7 +7831,7 @@
         <v>0.5</v>
       </c>
       <c r="W32" s="32" t="n">
-        <v>0.08982707293651104</v>
+        <v>9.069310059722595</v>
       </c>
       <c r="X32" s="32" t="n">
         <v>89</v>
@@ -7121,22 +7870,22 @@
         </is>
       </c>
       <c r="AH32" s="33" t="n">
-        <v/>
+        <v>317.5376230100137</v>
       </c>
       <c r="AI32" s="34" t="n">
         <v>220</v>
       </c>
       <c r="AJ32" s="33" t="n">
-        <v/>
+        <v>396.9220287625171</v>
       </c>
       <c r="AK32" s="35" t="n">
-        <v/>
+        <v>48.54405016603422</v>
       </c>
       <c r="AL32" s="39" t="n">
-        <v>0.04152542372881356</v>
+        <v>10</v>
       </c>
       <c r="AM32" s="36" t="n">
-        <v>41525.42372881356</v>
+        <v>100000</v>
       </c>
       <c r="AN32" s="32" t="inlineStr">
         <is>
@@ -7187,11 +7936,35 @@
         <v>13.51000014923837</v>
       </c>
       <c r="AX32" s="38" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="AY32" s="38">
-        <f>IFERROR(IF(OR(T32="",T32=0,AW32="",T32-AX32&lt;3),"N/A",ROUND((1-(AX32/T32))*100/(Dashboard!$B$14-AX32),1)),"N/A")</f>
-        <v/>
+        <v>21.6306065692</v>
+      </c>
+      <c r="AY32" s="38" t="n">
+        <v>29.37986889433879</v>
+      </c>
+      <c r="BA32" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="BC32" t="n">
+        <v>15.117691</v>
+      </c>
+      <c r="BE32" t="n">
+        <v>100</v>
+      </c>
+      <c r="BF32" t="n">
+        <v>19.50281827459328</v>
+      </c>
+      <c r="BG32" t="n">
+        <v>100</v>
+      </c>
+      <c r="BI32" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="BJ32" t="inlineStr">
+        <is>
+          <t>Strong Buy</t>
+        </is>
       </c>
     </row>
     <row r="33" ht="15" customHeight="1" s="24">
@@ -7219,7 +7992,7 @@
         </is>
       </c>
       <c r="F33" s="32" t="n">
-        <v>743787724800</v>
+        <v>741589778432</v>
       </c>
       <c r="G33" s="32" t="inlineStr">
         <is>
@@ -7232,16 +8005,16 @@
         </is>
       </c>
       <c r="I33" s="32" t="n">
-        <v>24.5</v>
+        <v>79.5</v>
       </c>
       <c r="J33" s="32" t="n">
-        <v>25.64047280308206</v>
+        <v>28.98083917636309</v>
       </c>
       <c r="K33" s="32" t="n">
         <v>75</v>
       </c>
       <c r="L33" s="32" t="n">
-        <v>60</v>
+        <v>100</v>
       </c>
       <c r="M33" s="32" t="inlineStr">
         <is>
@@ -7268,7 +8041,7 @@
         <v>0.28</v>
       </c>
       <c r="S33" s="32" t="n">
-        <v>9.183434007036881</v>
+        <v>9.15840700536306</v>
       </c>
       <c r="T33" s="32" t="n">
         <v>0.2186417857536935</v>
@@ -7280,7 +8053,7 @@
         <v>0.13</v>
       </c>
       <c r="W33" s="32" t="n">
-        <v>0.0226343725290097</v>
+        <v>2.269622504100635</v>
       </c>
       <c r="X33" s="32" t="n">
         <v>60.7</v>
@@ -7319,22 +8092,22 @@
         </is>
       </c>
       <c r="AH33" s="33" t="n">
-        <v>49.10384585352765</v>
+        <v>53.90839838710311</v>
       </c>
       <c r="AI33" s="34" t="n">
         <v>88</v>
       </c>
       <c r="AJ33" s="33" t="n">
-        <v>61.37980731690956</v>
+        <v>67.38549798387888</v>
       </c>
       <c r="AK33" s="35" t="n">
-        <v>-0.3783034469822046</v>
+        <v>-25.17530110140265</v>
       </c>
       <c r="AL33" s="39" t="n">
-        <v>0.04152542372881356</v>
+        <v>4.057097766669344</v>
       </c>
       <c r="AM33" s="36" t="n">
-        <v>41525.42372881356</v>
+        <v>40570.97766669344</v>
       </c>
       <c r="AN33" s="32" t="inlineStr">
         <is>
@@ -7382,13 +8155,38 @@
         </is>
       </c>
       <c r="AW33" s="37" t="n">
-        <v>8.439999732633577</v>
+        <v>8.470000583410828</v>
       </c>
       <c r="AX33" s="38" t="n">
-        <v>0.1</v>
+        <v>13.7094084</v>
       </c>
       <c r="AY33" s="38" t="n">
-        <v>7.246730497864174</v>
+        <v>7.955784885936112</v>
+      </c>
+      <c r="BA33" t="n">
+        <v>4.11</v>
+      </c>
+      <c r="BC33" t="n">
+        <v>9.958677</v>
+      </c>
+      <c r="BE33" t="n">
+        <v>100</v>
+      </c>
+      <c r="BF33" t="n">
+        <v>51.28094560616412</v>
+      </c>
+      <c r="BG33" t="n">
+        <v>100</v>
+      </c>
+      <c r="BI33" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="BJ33" t="inlineStr">
+        <is>
+          <t>Avoid</t>
+        </is>
       </c>
     </row>
     <row r="34" ht="15" customHeight="1" s="24">
@@ -7416,7 +8214,7 @@
         </is>
       </c>
       <c r="F34" s="32" t="n">
-        <v>60152782848</v>
+        <v>60310396928</v>
       </c>
       <c r="G34" s="32" t="inlineStr">
         <is>
@@ -7429,16 +8227,16 @@
         </is>
       </c>
       <c r="I34" s="32" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="J34" s="32" t="n">
-        <v>26.3323261370476</v>
+        <v>2.506178142689238</v>
       </c>
       <c r="K34" s="32" t="n">
         <v>65</v>
       </c>
       <c r="L34" s="32" t="n">
-        <v>55</v>
+        <v>100</v>
       </c>
       <c r="M34" s="32" t="inlineStr">
         <is>
@@ -7465,7 +8263,7 @@
         <v>0.38</v>
       </c>
       <c r="S34" s="32" t="n">
-        <v>16.9108785824608</v>
+        <v>16.94821550386128</v>
       </c>
       <c r="T34" s="32" t="n">
         <v>0.2440495370342224</v>
@@ -7477,7 +8275,7 @@
         <v>0.6899999999999999</v>
       </c>
       <c r="W34" s="32" t="n">
-        <v>0.02570755202494456</v>
+        <v>2.565091828382087</v>
       </c>
       <c r="X34" s="32" t="n">
         <v>98</v>
@@ -7516,24 +8314,22 @@
         </is>
       </c>
       <c r="AH34" s="33" t="n">
-        <v/>
+        <v>440.7884818996416</v>
       </c>
       <c r="AI34" s="34" t="n">
         <v>670</v>
       </c>
       <c r="AJ34" s="33" t="n">
-        <v/>
+        <v>550.9856023745519</v>
       </c>
       <c r="AK34" s="35" t="n">
-        <v/>
-      </c>
-      <c r="AL34" s="39">
-        <f>IF(H34="Fail","Not Eligible (Failed Gate)",IF(J34="","Pending Score",IF(J34&gt;=90,"10%",IF(J34&gt;=80,"7.5%",IF(J34&gt;=70,"5%","Watchlist only")))))</f>
-        <v/>
-      </c>
-      <c r="AM34" s="36">
-        <f>IFERROR(ROUND(VALUE(SUBSTITUTE(AL34,"%",""))/100*Dashboard!$B$11,0),"")</f>
-        <v/>
+        <v>-14.5855712525166</v>
+      </c>
+      <c r="AL34" s="39" t="n">
+        <v>0.3508459394051274</v>
+      </c>
+      <c r="AM34" s="36" t="n">
+        <v>3508.459394051274</v>
       </c>
       <c r="AN34" s="32" t="inlineStr">
         <is>
@@ -7584,11 +8380,35 @@
         <v>42.01999743489169</v>
       </c>
       <c r="AX34" s="38" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="AY34" s="38">
-        <f>IFERROR(IF(OR(T34="",T34=0,AW34="",T34-AX34&lt;3),"N/A",ROUND((1-(AX34/T34))*100/(Dashboard!$B$14-AX34),1)),"N/A")</f>
-        <v/>
+        <v>25</v>
+      </c>
+      <c r="AY34" s="38" t="n">
+        <v>13.11246078949433</v>
+      </c>
+      <c r="BA34" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="BC34" t="n">
+        <v>15.024987</v>
+      </c>
+      <c r="BE34" t="n">
+        <v>100</v>
+      </c>
+      <c r="BF34" t="n">
+        <v>92.6646522740952</v>
+      </c>
+      <c r="BG34" t="n">
+        <v>100</v>
+      </c>
+      <c r="BI34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="BJ34" t="inlineStr">
+        <is>
+          <t>Avoid</t>
+        </is>
       </c>
     </row>
     <row r="35" ht="15" customHeight="1" s="24">
@@ -7616,7 +8436,7 @@
         </is>
       </c>
       <c r="F35" s="32" t="n">
-        <v>102160392192</v>
+        <v>102407315456</v>
       </c>
       <c r="G35" s="32" t="inlineStr">
         <is>
@@ -7629,16 +8449,16 @@
         </is>
       </c>
       <c r="I35" s="39" t="n">
-        <v>24.5</v>
+        <v>89.5</v>
       </c>
       <c r="J35" s="39" t="n">
-        <v>24.64037817775813</v>
+        <v>100</v>
       </c>
       <c r="K35" s="32" t="n">
         <v>75</v>
       </c>
       <c r="L35" s="32" t="n">
-        <v>65</v>
+        <v>100</v>
       </c>
       <c r="M35" s="32" t="inlineStr">
         <is>
@@ -7665,7 +8485,7 @@
         <v>0.42</v>
       </c>
       <c r="S35" s="32" t="n">
-        <v>14.44058921336218</v>
+        <v>14.47463711254687</v>
       </c>
       <c r="T35" s="32" t="n">
         <v>0.2466884209645236</v>
@@ -7677,7 +8497,7 @@
         <v>0.1</v>
       </c>
       <c r="W35" s="32" t="n">
-        <v>0.07312791668370174</v>
+        <v>7.295590187493842</v>
       </c>
       <c r="X35" s="32" t="n">
         <v>36.7</v>
@@ -7716,22 +8536,22 @@
         </is>
       </c>
       <c r="AH35" s="33" t="n">
-        <v>195.7969908890691</v>
+        <v>331.4013486966001</v>
       </c>
       <c r="AI35" s="34" t="n">
         <v>262</v>
       </c>
       <c r="AJ35" s="33" t="n">
-        <v>244.7462386113364</v>
+        <v>414.25168587075</v>
       </c>
       <c r="AK35" s="35" t="n">
-        <v>-0.01431589473465903</v>
+        <v>39.92782443916396</v>
       </c>
       <c r="AL35" s="39" t="n">
-        <v>0.04152542372881356</v>
+        <v>10</v>
       </c>
       <c r="AM35" s="36" t="n">
-        <v>41525.42372881356</v>
+        <v>100000</v>
       </c>
       <c r="AN35" s="32" t="inlineStr">
         <is>
@@ -7779,13 +8599,38 @@
         </is>
       </c>
       <c r="AW35" s="37" t="n">
-        <v>16.63999909912754</v>
+        <v>16.64999882576862</v>
       </c>
       <c r="AX35" s="38" t="n">
-        <v>0.1</v>
+        <v>24.70821679857</v>
       </c>
       <c r="AY35" s="38" t="n">
-        <v>14.67303588796981</v>
+        <v>24.87998113337838</v>
+      </c>
+      <c r="BA35" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="BC35" t="n">
+        <v>14.945947</v>
+      </c>
+      <c r="BE35" t="n">
+        <v>100</v>
+      </c>
+      <c r="BF35" t="n">
+        <v>17.3384968041851</v>
+      </c>
+      <c r="BG35" t="n">
+        <v>100</v>
+      </c>
+      <c r="BI35" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="BJ35" t="inlineStr">
+        <is>
+          <t>Strong Buy</t>
+        </is>
       </c>
     </row>
     <row r="36" ht="15" customHeight="1" s="24">
@@ -7813,7 +8658,7 @@
         </is>
       </c>
       <c r="F36" s="32" t="n">
-        <v>137283305472</v>
+        <v>138175938560</v>
       </c>
       <c r="G36" s="32" t="inlineStr">
         <is>
@@ -7826,16 +8671,16 @@
         </is>
       </c>
       <c r="I36" s="32" t="n">
-        <v>24.5</v>
+        <v>89.5</v>
       </c>
       <c r="J36" s="32" t="n">
-        <v>24.50370402724242</v>
+        <v>69.17268154632724</v>
       </c>
       <c r="K36" s="32" t="n">
         <v>70</v>
       </c>
       <c r="L36" s="32" t="n">
-        <v>60</v>
+        <v>100</v>
       </c>
       <c r="M36" s="32" t="inlineStr">
         <is>
@@ -7862,7 +8707,7 @@
         <v>0.75</v>
       </c>
       <c r="S36" s="32" t="n">
-        <v>15.31756782196978</v>
+        <v>15.41945773654341</v>
       </c>
       <c r="T36" s="32" t="n">
         <v>0.2754079577698776</v>
@@ -7874,7 +8719,7 @@
         <v>0.13</v>
       </c>
       <c r="W36" s="32" t="n">
-        <v>0.05621314002546694</v>
+        <v>5.584169038482647</v>
       </c>
       <c r="X36" s="32" t="n">
         <v>23</v>
@@ -7913,22 +8758,22 @@
         </is>
       </c>
       <c r="AH36" s="33" t="n">
-        <v>853.72780863702</v>
+        <v>1466.272426201327</v>
       </c>
       <c r="AI36" s="34" t="n">
         <v>1400</v>
       </c>
       <c r="AJ36" s="33" t="n">
-        <v>1067.159760796275</v>
+        <v>1832.840532751659</v>
       </c>
       <c r="AK36" s="35" t="n">
-        <v>-0.3979162772093977</v>
+        <v>18.07797933485324</v>
       </c>
       <c r="AL36" s="32" t="n">
-        <v>0.04152542372881356</v>
+        <v>9.683650984303638</v>
       </c>
       <c r="AM36" s="36" t="n">
-        <v>41525.42372881356</v>
+        <v>96836.50984303637</v>
       </c>
       <c r="AN36" s="32" t="inlineStr">
         <is>
@@ -7979,10 +8824,35 @@
         <v>74.91999636197578</v>
       </c>
       <c r="AX36" s="38" t="n">
-        <v>0.1</v>
+        <v>25</v>
       </c>
       <c r="AY36" s="38" t="n">
-        <v>13.99920977038272</v>
+        <v>24.46396866993672</v>
+      </c>
+      <c r="BA36" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="BC36" t="n">
+        <v>20.041378</v>
+      </c>
+      <c r="BE36" t="n">
+        <v>100</v>
+      </c>
+      <c r="BF36" t="n">
+        <v>34.54502458660225</v>
+      </c>
+      <c r="BG36" t="n">
+        <v>100</v>
+      </c>
+      <c r="BI36" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="BJ36" t="inlineStr">
+        <is>
+          <t>Buy</t>
+        </is>
       </c>
     </row>
     <row r="37" ht="15" customHeight="1" s="24">
@@ -8010,7 +8880,7 @@
         </is>
       </c>
       <c r="F37" s="32" t="n">
-        <v>82366799872</v>
+        <v>82551750656</v>
       </c>
       <c r="G37" s="32" t="inlineStr">
         <is>
@@ -8023,16 +8893,16 @@
         </is>
       </c>
       <c r="I37" s="32" t="n">
-        <v>27.5</v>
+        <v>58</v>
       </c>
       <c r="J37" s="32" t="n">
-        <v>20</v>
+        <v>20.73847616194933</v>
       </c>
       <c r="K37" s="32" t="n">
         <v>35</v>
       </c>
       <c r="L37" s="32" t="n">
-        <v>35</v>
+        <v>100</v>
       </c>
       <c r="M37" s="32" t="inlineStr">
         <is>
@@ -8059,7 +8929,7 @@
         <v>0.21</v>
       </c>
       <c r="S37" s="32" t="n">
-        <v>11.21278151111012</v>
+        <v>11.23864788538567</v>
       </c>
       <c r="T37" s="32" t="n">
         <v>0.2170396084430917</v>
@@ -8071,7 +8941,7 @@
         <v>0.1</v>
       </c>
       <c r="W37" s="32" t="n">
-        <v>0.01975709633694587</v>
+        <v>1.97116242789491</v>
       </c>
       <c r="X37" s="32" t="n">
         <v>13</v>
@@ -8110,22 +8980,22 @@
         </is>
       </c>
       <c r="AH37" s="33" t="n">
-        <v>432.0274064308372</v>
+        <v>521.3427252991762</v>
       </c>
       <c r="AI37" s="34" t="n">
         <v>885</v>
       </c>
       <c r="AJ37" s="33" t="n">
-        <v>540.0342580385465</v>
+        <v>651.6784066239702</v>
       </c>
       <c r="AK37" s="35" t="n">
-        <v>-0.6905408988605972</v>
+        <v>-40.40667769554791</v>
       </c>
       <c r="AL37" s="32" t="n">
-        <v>0.04661016949152542</v>
+        <v>2.903229434066677</v>
       </c>
       <c r="AM37" s="36" t="n">
-        <v>46610.16949152543</v>
+        <v>29032.29434066677</v>
       </c>
       <c r="AN37" s="32" t="inlineStr">
         <is>
@@ -8176,10 +9046,35 @@
         <v>75.489992439011</v>
       </c>
       <c r="AX37" s="38" t="n">
-        <v>0.1</v>
+        <v>20.316037</v>
       </c>
       <c r="AY37" s="38" t="n">
-        <v>7.155614920346449</v>
+        <v>8.63264547124083</v>
+      </c>
+      <c r="BA37" t="n">
+        <v>1.95</v>
+      </c>
+      <c r="BC37" t="n">
+        <v>12.120811</v>
+      </c>
+      <c r="BE37" t="n">
+        <v>100</v>
+      </c>
+      <c r="BF37" t="n">
+        <v>40</v>
+      </c>
+      <c r="BG37" t="n">
+        <v>100</v>
+      </c>
+      <c r="BI37" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="BJ37" t="inlineStr">
+        <is>
+          <t>Avoid</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>